<commit_message>
Atualização automática LIRAa 2026-08-04 17:24 UTC
</commit_message>
<xml_diff>
--- a/data/LIRA_COMPLETO_latest.xlsx
+++ b/data/LIRA_COMPLETO_latest.xlsx
@@ -2594,13 +2594,13 @@
         <v>0</v>
       </c>
       <c r="C12" t="n">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="D12" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E12" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F12" t="n">
         <v>0</v>
@@ -2609,7 +2609,7 @@
         <v>0</v>
       </c>
       <c r="H12" t="n">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="I12" t="n">
         <v>0</v>
@@ -2676,13 +2676,13 @@
         <v>3</v>
       </c>
       <c r="C13" t="n">
-        <v>63</v>
+        <v>68</v>
       </c>
       <c r="D13" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="E13" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="F13" t="n">
         <v>3</v>
@@ -2691,7 +2691,7 @@
         <v>0</v>
       </c>
       <c r="H13" t="n">
-        <v>91</v>
+        <v>99</v>
       </c>
       <c r="I13" t="n">
         <v>0</v>
@@ -7214,13 +7214,13 @@
         <v>0</v>
       </c>
       <c r="C24" t="n">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="D24" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E24" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F24" t="n">
         <v>0</v>
@@ -7229,7 +7229,7 @@
         <v>0</v>
       </c>
       <c r="H24" t="n">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="I24" t="n">
         <v>0</v>
@@ -9346,13 +9346,13 @@
         <v>18</v>
       </c>
       <c r="C50" t="n">
-        <v>378</v>
+        <v>383</v>
       </c>
       <c r="D50" t="n">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="E50" t="n">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="F50" t="n">
         <v>36</v>
@@ -9361,7 +9361,7 @@
         <v>0</v>
       </c>
       <c r="H50" t="n">
-        <v>630</v>
+        <v>638</v>
       </c>
       <c r="I50" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Atualização automática LIRAa 2026-08-04 17:51 UTC
</commit_message>
<xml_diff>
--- a/data/LIRA_COMPLETO_latest.xlsx
+++ b/data/LIRA_COMPLETO_latest.xlsx
@@ -3803,10 +3803,10 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C13" t="n">
-        <v>13</v>
+        <v>26</v>
       </c>
       <c r="D13" t="n">
         <v>2</v>
@@ -3821,7 +3821,7 @@
         <v>0</v>
       </c>
       <c r="H13" t="n">
-        <v>20</v>
+        <v>33</v>
       </c>
       <c r="I13" t="n">
         <v>0</v>
@@ -3967,10 +3967,10 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C15" t="n">
-        <v>136</v>
+        <v>149</v>
       </c>
       <c r="D15" t="n">
         <v>9</v>
@@ -3985,7 +3985,7 @@
         <v>0</v>
       </c>
       <c r="H15" t="n">
-        <v>208</v>
+        <v>221</v>
       </c>
       <c r="I15" t="n">
         <v>0</v>
@@ -8195,10 +8195,10 @@
         </is>
       </c>
       <c r="B36" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C36" t="n">
-        <v>13</v>
+        <v>26</v>
       </c>
       <c r="D36" t="n">
         <v>2</v>
@@ -8213,7 +8213,7 @@
         <v>0</v>
       </c>
       <c r="H36" t="n">
-        <v>20</v>
+        <v>33</v>
       </c>
       <c r="I36" t="n">
         <v>0</v>
@@ -9343,10 +9343,10 @@
         </is>
       </c>
       <c r="B50" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C50" t="n">
-        <v>383</v>
+        <v>396</v>
       </c>
       <c r="D50" t="n">
         <v>40</v>
@@ -9361,7 +9361,7 @@
         <v>0</v>
       </c>
       <c r="H50" t="n">
-        <v>638</v>
+        <v>651</v>
       </c>
       <c r="I50" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Atualização automática LIRAa 2026-08-04 18:58 UTC
</commit_message>
<xml_diff>
--- a/data/LIRA_COMPLETO_latest.xlsx
+++ b/data/LIRA_COMPLETO_latest.xlsx
@@ -665,10 +665,10 @@
         <v>0</v>
       </c>
       <c r="J3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L3" t="n">
         <v>0</v>
@@ -683,7 +683,7 @@
         <v>0</v>
       </c>
       <c r="P3" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="Q3" t="n">
         <v>0</v>
@@ -692,13 +692,13 @@
         <v>0</v>
       </c>
       <c r="S3" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="T3" t="n">
         <v>0</v>
       </c>
       <c r="U3" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="V3" t="n">
         <v>0</v>
@@ -890,22 +890,22 @@
         <v>0</v>
       </c>
       <c r="C6" t="n">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="D6" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G6" t="n">
         <v>0</v>
       </c>
       <c r="H6" t="n">
-        <v>23</v>
+        <v>34</v>
       </c>
       <c r="I6" t="n">
         <v>0</v>
@@ -1546,31 +1546,31 @@
         <v>4</v>
       </c>
       <c r="C14" t="n">
-        <v>90</v>
+        <v>98</v>
       </c>
       <c r="D14" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="E14" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="F14" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="G14" t="n">
         <v>0</v>
       </c>
       <c r="H14" t="n">
-        <v>176</v>
+        <v>187</v>
       </c>
       <c r="I14" t="n">
         <v>0</v>
       </c>
       <c r="J14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L14" t="n">
         <v>0</v>
@@ -1585,7 +1585,7 @@
         <v>0</v>
       </c>
       <c r="P14" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="Q14" t="n">
         <v>0</v>
@@ -1594,13 +1594,13 @@
         <v>0</v>
       </c>
       <c r="S14" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="T14" t="n">
         <v>0</v>
       </c>
       <c r="U14" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="V14" t="n">
         <v>0</v>
@@ -5513,10 +5513,10 @@
         <v>0</v>
       </c>
       <c r="J3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L3" t="n">
         <v>0</v>
@@ -5531,7 +5531,7 @@
         <v>0</v>
       </c>
       <c r="P3" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="Q3" t="n">
         <v>0</v>
@@ -5540,13 +5540,13 @@
         <v>0</v>
       </c>
       <c r="S3" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="T3" t="n">
         <v>0</v>
       </c>
       <c r="U3" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="V3" t="n">
         <v>0</v>
@@ -5738,22 +5738,22 @@
         <v>0</v>
       </c>
       <c r="C6" t="n">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="D6" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G6" t="n">
         <v>0</v>
       </c>
       <c r="H6" t="n">
-        <v>23</v>
+        <v>34</v>
       </c>
       <c r="I6" t="n">
         <v>0</v>
@@ -9346,32 +9346,32 @@
         <v>19</v>
       </c>
       <c r="C50" t="n">
-        <v>396</v>
+        <v>404</v>
       </c>
       <c r="D50" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="E50" t="n">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="F50" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="G50" t="n">
         <v>0</v>
       </c>
       <c r="H50" t="n">
-        <v>651</v>
+        <v>662</v>
       </c>
       <c r="I50" t="n">
         <v>0</v>
       </c>
       <c r="J50" t="n">
+        <v>3</v>
+      </c>
+      <c r="K50" t="n">
         <v>2</v>
       </c>
-      <c r="K50" t="n">
-        <v>1</v>
-      </c>
       <c r="L50" t="n">
         <v>0</v>
       </c>
@@ -9385,7 +9385,7 @@
         <v>0</v>
       </c>
       <c r="P50" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="Q50" t="n">
         <v>3</v>
@@ -9394,13 +9394,13 @@
         <v>0</v>
       </c>
       <c r="S50" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="T50" t="n">
         <v>0</v>
       </c>
       <c r="U50" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="V50" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Atualização automática LIRAa 2026-08-04 19:37 UTC
</commit_message>
<xml_diff>
--- a/data/LIRA_COMPLETO_latest.xlsx
+++ b/data/LIRA_COMPLETO_latest.xlsx
@@ -1054,13 +1054,13 @@
         <v>0</v>
       </c>
       <c r="C8" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D8" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E8" t="n">
-        <v>19</v>
+        <v>29</v>
       </c>
       <c r="F8" t="n">
         <v>2</v>
@@ -1069,7 +1069,7 @@
         <v>0</v>
       </c>
       <c r="H8" t="n">
-        <v>28</v>
+        <v>40</v>
       </c>
       <c r="I8" t="n">
         <v>0</v>
@@ -1546,13 +1546,13 @@
         <v>4</v>
       </c>
       <c r="C14" t="n">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="D14" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E14" t="n">
-        <v>58</v>
+        <v>68</v>
       </c>
       <c r="F14" t="n">
         <v>14</v>
@@ -1561,7 +1561,7 @@
         <v>0</v>
       </c>
       <c r="H14" t="n">
-        <v>187</v>
+        <v>199</v>
       </c>
       <c r="I14" t="n">
         <v>0</v>
@@ -5100,13 +5100,13 @@
         <v>0</v>
       </c>
       <c r="C13" t="n">
+        <v>26</v>
+      </c>
+      <c r="D13" t="n">
+        <v>2</v>
+      </c>
+      <c r="E13" t="n">
         <v>8</v>
-      </c>
-      <c r="D13" t="n">
-        <v>1</v>
-      </c>
-      <c r="E13" t="n">
-        <v>5</v>
       </c>
       <c r="F13" t="n">
         <v>2</v>
@@ -5115,7 +5115,7 @@
         <v>0</v>
       </c>
       <c r="H13" t="n">
-        <v>16</v>
+        <v>38</v>
       </c>
       <c r="I13" t="n">
         <v>0</v>
@@ -5182,13 +5182,13 @@
         <v>4</v>
       </c>
       <c r="C14" t="n">
-        <v>89</v>
+        <v>107</v>
       </c>
       <c r="D14" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E14" t="n">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="F14" t="n">
         <v>9</v>
@@ -5197,7 +5197,7 @@
         <v>0</v>
       </c>
       <c r="H14" t="n">
-        <v>155</v>
+        <v>177</v>
       </c>
       <c r="I14" t="n">
         <v>0</v>
@@ -5902,13 +5902,13 @@
         <v>0</v>
       </c>
       <c r="C8" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D8" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E8" t="n">
-        <v>19</v>
+        <v>29</v>
       </c>
       <c r="F8" t="n">
         <v>2</v>
@@ -5917,7 +5917,7 @@
         <v>0</v>
       </c>
       <c r="H8" t="n">
-        <v>28</v>
+        <v>40</v>
       </c>
       <c r="I8" t="n">
         <v>0</v>
@@ -9264,13 +9264,13 @@
         <v>0</v>
       </c>
       <c r="C49" t="n">
+        <v>26</v>
+      </c>
+      <c r="D49" t="n">
+        <v>2</v>
+      </c>
+      <c r="E49" t="n">
         <v>8</v>
-      </c>
-      <c r="D49" t="n">
-        <v>1</v>
-      </c>
-      <c r="E49" t="n">
-        <v>5</v>
       </c>
       <c r="F49" t="n">
         <v>2</v>
@@ -9279,7 +9279,7 @@
         <v>0</v>
       </c>
       <c r="H49" t="n">
-        <v>16</v>
+        <v>38</v>
       </c>
       <c r="I49" t="n">
         <v>0</v>
@@ -9346,13 +9346,13 @@
         <v>19</v>
       </c>
       <c r="C50" t="n">
-        <v>404</v>
+        <v>423</v>
       </c>
       <c r="D50" t="n">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="E50" t="n">
-        <v>180</v>
+        <v>193</v>
       </c>
       <c r="F50" t="n">
         <v>37</v>
@@ -9361,7 +9361,7 @@
         <v>0</v>
       </c>
       <c r="H50" t="n">
-        <v>662</v>
+        <v>696</v>
       </c>
       <c r="I50" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Atualização automática LIRAa 2026-08-04 19:44 UTC
</commit_message>
<xml_diff>
--- a/data/LIRA_COMPLETO_latest.xlsx
+++ b/data/LIRA_COMPLETO_latest.xlsx
@@ -3143,29 +3143,29 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>AREA_1445</t>
+          <t>426 - NOVA PONTA PORÃ - ESTRATO 3</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C5" t="n">
-        <v>0</v>
+        <v>21</v>
       </c>
       <c r="D5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E5" t="n">
-        <v>0</v>
+        <v>19</v>
       </c>
       <c r="F5" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G5" t="n">
         <v>0</v>
       </c>
       <c r="H5" t="n">
-        <v>0</v>
+        <v>43</v>
       </c>
       <c r="I5" t="n">
         <v>0</v>
@@ -3967,25 +3967,25 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C15" t="n">
-        <v>149</v>
+        <v>170</v>
       </c>
       <c r="D15" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E15" t="n">
-        <v>52</v>
+        <v>71</v>
       </c>
       <c r="F15" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="G15" t="n">
         <v>0</v>
       </c>
       <c r="H15" t="n">
-        <v>221</v>
+        <v>264</v>
       </c>
       <c r="I15" t="n">
         <v>0</v>
@@ -7535,29 +7535,29 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>AREA_1445</t>
+          <t>426 - NOVA PONTA PORÃ - ESTRATO 3</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C28" t="n">
-        <v>0</v>
+        <v>21</v>
       </c>
       <c r="D28" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E28" t="n">
-        <v>0</v>
+        <v>19</v>
       </c>
       <c r="F28" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G28" t="n">
         <v>0</v>
       </c>
       <c r="H28" t="n">
-        <v>0</v>
+        <v>43</v>
       </c>
       <c r="I28" t="n">
         <v>0</v>
@@ -9343,25 +9343,25 @@
         </is>
       </c>
       <c r="B50" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C50" t="n">
-        <v>423</v>
+        <v>444</v>
       </c>
       <c r="D50" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="E50" t="n">
-        <v>193</v>
+        <v>212</v>
       </c>
       <c r="F50" t="n">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="G50" t="n">
         <v>0</v>
       </c>
       <c r="H50" t="n">
-        <v>696</v>
+        <v>739</v>
       </c>
       <c r="I50" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Atualização automática LIRAa 2026-08-04 20:12 UTC
</commit_message>
<xml_diff>
--- a/data/LIRA_COMPLETO_latest.xlsx
+++ b/data/LIRA_COMPLETO_latest.xlsx
@@ -3639,16 +3639,16 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C11" t="n">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="D11" t="n">
         <v>1</v>
       </c>
       <c r="E11" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="F11" t="n">
         <v>2</v>
@@ -3657,7 +3657,7 @@
         <v>0</v>
       </c>
       <c r="H11" t="n">
-        <v>25</v>
+        <v>34</v>
       </c>
       <c r="I11" t="n">
         <v>0</v>
@@ -3967,16 +3967,16 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="C15" t="n">
-        <v>170</v>
+        <v>175</v>
       </c>
       <c r="D15" t="n">
         <v>10</v>
       </c>
       <c r="E15" t="n">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="F15" t="n">
         <v>13</v>
@@ -3985,7 +3985,7 @@
         <v>0</v>
       </c>
       <c r="H15" t="n">
-        <v>264</v>
+        <v>273</v>
       </c>
       <c r="I15" t="n">
         <v>0</v>
@@ -8031,16 +8031,16 @@
         </is>
       </c>
       <c r="B34" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C34" t="n">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="D34" t="n">
         <v>1</v>
       </c>
       <c r="E34" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="F34" t="n">
         <v>2</v>
@@ -8049,7 +8049,7 @@
         <v>0</v>
       </c>
       <c r="H34" t="n">
-        <v>25</v>
+        <v>34</v>
       </c>
       <c r="I34" t="n">
         <v>0</v>
@@ -9343,16 +9343,16 @@
         </is>
       </c>
       <c r="B50" t="n">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="C50" t="n">
-        <v>444</v>
+        <v>449</v>
       </c>
       <c r="D50" t="n">
         <v>44</v>
       </c>
       <c r="E50" t="n">
-        <v>212</v>
+        <v>216</v>
       </c>
       <c r="F50" t="n">
         <v>39</v>
@@ -9361,7 +9361,7 @@
         <v>0</v>
       </c>
       <c r="H50" t="n">
-        <v>739</v>
+        <v>748</v>
       </c>
       <c r="I50" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Atualização automática LIRAa 2026-08-04 23:22 UTC
</commit_message>
<xml_diff>
--- a/data/LIRA_COMPLETO_latest.xlsx
+++ b/data/LIRA_COMPLETO_latest.xlsx
@@ -644,13 +644,13 @@
         <v>4</v>
       </c>
       <c r="C3" t="n">
-        <v>20</v>
+        <v>33</v>
       </c>
       <c r="D3" t="n">
         <v>1</v>
       </c>
       <c r="E3" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="F3" t="n">
         <v>1</v>
@@ -659,7 +659,7 @@
         <v>0</v>
       </c>
       <c r="H3" t="n">
-        <v>30</v>
+        <v>44</v>
       </c>
       <c r="I3" t="n">
         <v>0</v>
@@ -801,29 +801,29 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>AREA_1239</t>
+          <t>403 - JARDIM UNIVERSITARIO - ESTRATO 1</t>
         </is>
       </c>
       <c r="B5" t="n">
         <v>0</v>
       </c>
       <c r="C5" t="n">
-        <v>0</v>
+        <v>19</v>
       </c>
       <c r="D5" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="E5" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="F5" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="G5" t="n">
         <v>0</v>
       </c>
       <c r="H5" t="n">
-        <v>0</v>
+        <v>32</v>
       </c>
       <c r="I5" t="n">
         <v>0</v>
@@ -1129,29 +1129,29 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>AREA_1416</t>
+          <t>407 - BAIRRO MOOCA - ESTRATO 1</t>
         </is>
       </c>
       <c r="B9" t="n">
         <v>0</v>
       </c>
       <c r="C9" t="n">
-        <v>0</v>
+        <v>14</v>
       </c>
       <c r="D9" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E9" t="n">
-        <v>0</v>
+        <v>18</v>
       </c>
       <c r="F9" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G9" t="n">
         <v>0</v>
       </c>
       <c r="H9" t="n">
-        <v>0</v>
+        <v>36</v>
       </c>
       <c r="I9" t="n">
         <v>0</v>
@@ -1221,7 +1221,7 @@
         <v>12</v>
       </c>
       <c r="D10" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E10" t="n">
         <v>9</v>
@@ -1233,7 +1233,7 @@
         <v>0</v>
       </c>
       <c r="H10" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="I10" t="n">
         <v>0</v>
@@ -1300,22 +1300,22 @@
         <v>0</v>
       </c>
       <c r="C11" t="n">
-        <v>6</v>
+        <v>18</v>
       </c>
       <c r="D11" t="n">
         <v>1</v>
       </c>
       <c r="E11" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="F11" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G11" t="n">
         <v>0</v>
       </c>
       <c r="H11" t="n">
-        <v>12</v>
+        <v>28</v>
       </c>
       <c r="I11" t="n">
         <v>0</v>
@@ -1464,22 +1464,22 @@
         <v>0</v>
       </c>
       <c r="C13" t="n">
-        <v>11</v>
+        <v>19</v>
       </c>
       <c r="D13" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E13" t="n">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="F13" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G13" t="n">
         <v>0</v>
       </c>
       <c r="H13" t="n">
-        <v>26</v>
+        <v>41</v>
       </c>
       <c r="I13" t="n">
         <v>0</v>
@@ -1546,22 +1546,22 @@
         <v>4</v>
       </c>
       <c r="C14" t="n">
-        <v>99</v>
+        <v>165</v>
       </c>
       <c r="D14" t="n">
-        <v>18</v>
+        <v>26</v>
       </c>
       <c r="E14" t="n">
-        <v>68</v>
+        <v>100</v>
       </c>
       <c r="F14" t="n">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="G14" t="n">
         <v>0</v>
       </c>
       <c r="H14" t="n">
-        <v>199</v>
+        <v>313</v>
       </c>
       <c r="I14" t="n">
         <v>0</v>
@@ -1774,7 +1774,7 @@
         <v>0</v>
       </c>
       <c r="C2" t="n">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="D2" t="n">
         <v>1</v>
@@ -1789,7 +1789,7 @@
         <v>0</v>
       </c>
       <c r="H2" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="I2" t="n">
         <v>0</v>
@@ -1849,29 +1849,29 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>AREA_1422</t>
+          <t>413 - BAIRRO DA GRANJA - ESTRATO 2</t>
         </is>
       </c>
       <c r="B3" t="n">
         <v>0</v>
       </c>
       <c r="C3" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="D3" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="E3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F3" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G3" t="n">
         <v>0</v>
       </c>
       <c r="H3" t="n">
-        <v>0</v>
+        <v>29</v>
       </c>
       <c r="I3" t="n">
         <v>0</v>
@@ -1938,22 +1938,22 @@
         <v>0</v>
       </c>
       <c r="C4" t="n">
-        <v>7</v>
+        <v>15</v>
       </c>
       <c r="D4" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="E4" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="F4" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="G4" t="n">
         <v>0</v>
       </c>
       <c r="H4" t="n">
-        <v>12</v>
+        <v>35</v>
       </c>
       <c r="I4" t="n">
         <v>0</v>
@@ -2095,29 +2095,29 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>AREA_1425</t>
+          <t>416 - CENTRO 2 - ESTRATO 2</t>
         </is>
       </c>
       <c r="B6" t="n">
         <v>0</v>
       </c>
       <c r="C6" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D6" t="n">
-        <v>0</v>
+        <v>18</v>
       </c>
       <c r="E6" t="n">
         <v>0</v>
       </c>
       <c r="F6" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G6" t="n">
         <v>0</v>
       </c>
       <c r="H6" t="n">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="I6" t="n">
         <v>0</v>
@@ -2177,29 +2177,29 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>AREA_1426</t>
+          <t>417 - CENTRO 3 - ESTRATO 2</t>
         </is>
       </c>
       <c r="B7" t="n">
         <v>0</v>
       </c>
       <c r="C7" t="n">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="D7" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="E7" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F7" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="G7" t="n">
         <v>0</v>
       </c>
       <c r="H7" t="n">
-        <v>0</v>
+        <v>23</v>
       </c>
       <c r="I7" t="n">
         <v>0</v>
@@ -2259,20 +2259,20 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>AREA_1427</t>
+          <t>418 - CENTRO 4 - ESTRATO 2</t>
         </is>
       </c>
       <c r="B8" t="n">
         <v>0</v>
       </c>
       <c r="C8" t="n">
-        <v>0</v>
+        <v>19</v>
       </c>
       <c r="D8" t="n">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="E8" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F8" t="n">
         <v>0</v>
@@ -2281,7 +2281,7 @@
         <v>0</v>
       </c>
       <c r="H8" t="n">
-        <v>0</v>
+        <v>32</v>
       </c>
       <c r="I8" t="n">
         <v>0</v>
@@ -2345,25 +2345,25 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C9" t="n">
+        <v>9</v>
+      </c>
+      <c r="D9" t="n">
         <v>5</v>
       </c>
-      <c r="D9" t="n">
-        <v>1</v>
-      </c>
       <c r="E9" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F9" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G9" t="n">
         <v>0</v>
       </c>
       <c r="H9" t="n">
-        <v>9</v>
+        <v>20</v>
       </c>
       <c r="I9" t="n">
         <v>0</v>
@@ -2427,16 +2427,16 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C10" t="n">
-        <v>16</v>
+        <v>27</v>
       </c>
       <c r="D10" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E10" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F10" t="n">
         <v>0</v>
@@ -2445,7 +2445,7 @@
         <v>0</v>
       </c>
       <c r="H10" t="n">
-        <v>20</v>
+        <v>35</v>
       </c>
       <c r="I10" t="n">
         <v>0</v>
@@ -2512,7 +2512,7 @@
         <v>0</v>
       </c>
       <c r="C11" t="n">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="D11" t="n">
         <v>2</v>
@@ -2521,13 +2521,13 @@
         <v>5</v>
       </c>
       <c r="F11" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G11" t="n">
         <v>0</v>
       </c>
       <c r="H11" t="n">
-        <v>26</v>
+        <v>33</v>
       </c>
       <c r="I11" t="n">
         <v>0</v>
@@ -2594,10 +2594,10 @@
         <v>0</v>
       </c>
       <c r="C12" t="n">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="D12" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E12" t="n">
         <v>3</v>
@@ -2609,7 +2609,7 @@
         <v>0</v>
       </c>
       <c r="H12" t="n">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="I12" t="n">
         <v>0</v>
@@ -2673,25 +2673,25 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="C13" t="n">
-        <v>68</v>
+        <v>166</v>
       </c>
       <c r="D13" t="n">
-        <v>10</v>
+        <v>62</v>
       </c>
       <c r="E13" t="n">
-        <v>18</v>
+        <v>31</v>
       </c>
       <c r="F13" t="n">
-        <v>3</v>
+        <v>21</v>
       </c>
       <c r="G13" t="n">
         <v>0</v>
       </c>
       <c r="H13" t="n">
-        <v>99</v>
+        <v>280</v>
       </c>
       <c r="I13" t="n">
         <v>0</v>
@@ -2904,7 +2904,7 @@
         <v>1</v>
       </c>
       <c r="C2" t="n">
-        <v>11</v>
+        <v>24</v>
       </c>
       <c r="D2" t="n">
         <v>0</v>
@@ -2913,13 +2913,13 @@
         <v>1</v>
       </c>
       <c r="F2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G2" t="n">
         <v>0</v>
       </c>
       <c r="H2" t="n">
-        <v>13</v>
+        <v>27</v>
       </c>
       <c r="I2" t="n">
         <v>0</v>
@@ -2983,16 +2983,16 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C3" t="n">
-        <v>11</v>
+        <v>22</v>
       </c>
       <c r="D3" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E3" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="F3" t="n">
         <v>1</v>
@@ -3001,7 +3001,7 @@
         <v>0</v>
       </c>
       <c r="H3" t="n">
-        <v>18</v>
+        <v>34</v>
       </c>
       <c r="I3" t="n">
         <v>0</v>
@@ -3229,17 +3229,17 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C6" t="n">
+        <v>21</v>
+      </c>
+      <c r="D6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E6" t="n">
         <v>15</v>
       </c>
-      <c r="D6" t="n">
-        <v>0</v>
-      </c>
-      <c r="E6" t="n">
-        <v>8</v>
-      </c>
       <c r="F6" t="n">
         <v>1</v>
       </c>
@@ -3247,7 +3247,7 @@
         <v>0</v>
       </c>
       <c r="H6" t="n">
-        <v>24</v>
+        <v>37</v>
       </c>
       <c r="I6" t="n">
         <v>0</v>
@@ -3314,22 +3314,22 @@
         <v>1</v>
       </c>
       <c r="C7" t="n">
-        <v>13</v>
+        <v>25</v>
       </c>
       <c r="D7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E7" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="F7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G7" t="n">
         <v>0</v>
       </c>
       <c r="H7" t="n">
-        <v>20</v>
+        <v>36</v>
       </c>
       <c r="I7" t="n">
         <v>0</v>
@@ -3393,25 +3393,25 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C8" t="n">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="D8" t="n">
         <v>0</v>
       </c>
       <c r="E8" t="n">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="F8" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G8" t="n">
         <v>0</v>
       </c>
       <c r="H8" t="n">
-        <v>16</v>
+        <v>31</v>
       </c>
       <c r="I8" t="n">
         <v>0</v>
@@ -3478,13 +3478,13 @@
         <v>0</v>
       </c>
       <c r="C9" t="n">
-        <v>9</v>
+        <v>21</v>
       </c>
       <c r="D9" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E9" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="F9" t="n">
         <v>1</v>
@@ -3493,7 +3493,7 @@
         <v>0</v>
       </c>
       <c r="H9" t="n">
-        <v>17</v>
+        <v>32</v>
       </c>
       <c r="I9" t="n">
         <v>0</v>
@@ -3553,29 +3553,29 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>AREA_1450</t>
+          <t>431 - PANAMBI - ESTRATO 3</t>
         </is>
       </c>
       <c r="B10" t="n">
         <v>0</v>
       </c>
       <c r="C10" t="n">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="D10" t="n">
         <v>0</v>
       </c>
       <c r="E10" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F10" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G10" t="n">
         <v>0</v>
       </c>
       <c r="H10" t="n">
-        <v>0</v>
+        <v>18</v>
       </c>
       <c r="I10" t="n">
         <v>0</v>
@@ -3888,13 +3888,13 @@
         <v>0</v>
       </c>
       <c r="C14" t="n">
-        <v>10</v>
+        <v>22</v>
       </c>
       <c r="D14" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E14" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="F14" t="n">
         <v>0</v>
@@ -3903,7 +3903,7 @@
         <v>0</v>
       </c>
       <c r="H14" t="n">
-        <v>19</v>
+        <v>35</v>
       </c>
       <c r="I14" t="n">
         <v>0</v>
@@ -3967,25 +3967,25 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="C15" t="n">
-        <v>175</v>
+        <v>259</v>
       </c>
       <c r="D15" t="n">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="E15" t="n">
-        <v>75</v>
+        <v>103</v>
       </c>
       <c r="F15" t="n">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="G15" t="n">
         <v>0</v>
       </c>
       <c r="H15" t="n">
-        <v>273</v>
+        <v>396</v>
       </c>
       <c r="I15" t="n">
         <v>0</v>
@@ -4362,13 +4362,13 @@
         <v>1</v>
       </c>
       <c r="C4" t="n">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="D4" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E4" t="n">
-        <v>8</v>
+        <v>17</v>
       </c>
       <c r="F4" t="n">
         <v>2</v>
@@ -4377,7 +4377,7 @@
         <v>0</v>
       </c>
       <c r="H4" t="n">
-        <v>25</v>
+        <v>42</v>
       </c>
       <c r="I4" t="n">
         <v>0</v>
@@ -4526,13 +4526,13 @@
         <v>0</v>
       </c>
       <c r="C6" t="n">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="D6" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E6" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="F6" t="n">
         <v>0</v>
@@ -4541,7 +4541,7 @@
         <v>0</v>
       </c>
       <c r="H6" t="n">
-        <v>18</v>
+        <v>36</v>
       </c>
       <c r="I6" t="n">
         <v>0</v>
@@ -4601,29 +4601,29 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>AREA_1485</t>
+          <t>440 - JARDIM IBIRAPUERA - ESTRATO 4</t>
         </is>
       </c>
       <c r="B7" t="n">
         <v>0</v>
       </c>
       <c r="C7" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="D7" t="n">
         <v>0</v>
       </c>
       <c r="E7" t="n">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="F7" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G7" t="n">
         <v>0</v>
       </c>
       <c r="H7" t="n">
-        <v>0</v>
+        <v>21</v>
       </c>
       <c r="I7" t="n">
         <v>0</v>
@@ -4683,29 +4683,29 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>AREA_1486</t>
+          <t>441 - PARQUE DOS IPES - ESTRATO 4</t>
         </is>
       </c>
       <c r="B8" t="n">
         <v>0</v>
       </c>
       <c r="C8" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="D8" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E8" t="n">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="F8" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G8" t="n">
         <v>0</v>
       </c>
       <c r="H8" t="n">
-        <v>0</v>
+        <v>26</v>
       </c>
       <c r="I8" t="n">
         <v>0</v>
@@ -4769,10 +4769,10 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C9" t="n">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="D9" t="n">
         <v>0</v>
@@ -4787,7 +4787,7 @@
         <v>0</v>
       </c>
       <c r="H9" t="n">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="I9" t="n">
         <v>0</v>
@@ -4847,29 +4847,29 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>AREA_2596</t>
+          <t>446 - GUY VILELA - ESTRATO 4</t>
         </is>
       </c>
       <c r="B10" t="n">
         <v>0</v>
       </c>
       <c r="C10" t="n">
-        <v>0</v>
+        <v>21</v>
       </c>
       <c r="D10" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="E10" t="n">
-        <v>0</v>
+        <v>18</v>
       </c>
       <c r="F10" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="G10" t="n">
         <v>0</v>
       </c>
       <c r="H10" t="n">
-        <v>0</v>
+        <v>48</v>
       </c>
       <c r="I10" t="n">
         <v>0</v>
@@ -5018,13 +5018,13 @@
         <v>0</v>
       </c>
       <c r="C12" t="n">
-        <v>13</v>
+        <v>25</v>
       </c>
       <c r="D12" t="n">
         <v>0</v>
       </c>
       <c r="E12" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="F12" t="n">
         <v>1</v>
@@ -5033,7 +5033,7 @@
         <v>0</v>
       </c>
       <c r="H12" t="n">
-        <v>15</v>
+        <v>32</v>
       </c>
       <c r="I12" t="n">
         <v>0</v>
@@ -5179,25 +5179,25 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C14" t="n">
-        <v>107</v>
+        <v>180</v>
       </c>
       <c r="D14" t="n">
-        <v>6</v>
+        <v>14</v>
       </c>
       <c r="E14" t="n">
-        <v>55</v>
+        <v>115</v>
       </c>
       <c r="F14" t="n">
-        <v>9</v>
+        <v>20</v>
       </c>
       <c r="G14" t="n">
         <v>0</v>
       </c>
       <c r="H14" t="n">
-        <v>177</v>
+        <v>329</v>
       </c>
       <c r="I14" t="n">
         <v>0</v>
@@ -5492,13 +5492,13 @@
         <v>4</v>
       </c>
       <c r="C3" t="n">
-        <v>20</v>
+        <v>33</v>
       </c>
       <c r="D3" t="n">
         <v>1</v>
       </c>
       <c r="E3" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="F3" t="n">
         <v>1</v>
@@ -5507,7 +5507,7 @@
         <v>0</v>
       </c>
       <c r="H3" t="n">
-        <v>30</v>
+        <v>44</v>
       </c>
       <c r="I3" t="n">
         <v>0</v>
@@ -5649,29 +5649,29 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>AREA_1239</t>
+          <t>403 - JARDIM UNIVERSITARIO - ESTRATO 1</t>
         </is>
       </c>
       <c r="B5" t="n">
         <v>0</v>
       </c>
       <c r="C5" t="n">
-        <v>0</v>
+        <v>19</v>
       </c>
       <c r="D5" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="E5" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="F5" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="G5" t="n">
         <v>0</v>
       </c>
       <c r="H5" t="n">
-        <v>0</v>
+        <v>32</v>
       </c>
       <c r="I5" t="n">
         <v>0</v>
@@ -5977,29 +5977,29 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>AREA_1416</t>
+          <t>407 - BAIRRO MOOCA - ESTRATO 1</t>
         </is>
       </c>
       <c r="B9" t="n">
         <v>0</v>
       </c>
       <c r="C9" t="n">
-        <v>0</v>
+        <v>14</v>
       </c>
       <c r="D9" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E9" t="n">
-        <v>0</v>
+        <v>18</v>
       </c>
       <c r="F9" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G9" t="n">
         <v>0</v>
       </c>
       <c r="H9" t="n">
-        <v>0</v>
+        <v>36</v>
       </c>
       <c r="I9" t="n">
         <v>0</v>
@@ -6069,7 +6069,7 @@
         <v>12</v>
       </c>
       <c r="D10" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E10" t="n">
         <v>9</v>
@@ -6081,7 +6081,7 @@
         <v>0</v>
       </c>
       <c r="H10" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="I10" t="n">
         <v>0</v>
@@ -6148,22 +6148,22 @@
         <v>0</v>
       </c>
       <c r="C11" t="n">
-        <v>6</v>
+        <v>18</v>
       </c>
       <c r="D11" t="n">
         <v>1</v>
       </c>
       <c r="E11" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="F11" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G11" t="n">
         <v>0</v>
       </c>
       <c r="H11" t="n">
-        <v>12</v>
+        <v>28</v>
       </c>
       <c r="I11" t="n">
         <v>0</v>
@@ -6312,22 +6312,22 @@
         <v>0</v>
       </c>
       <c r="C13" t="n">
-        <v>11</v>
+        <v>19</v>
       </c>
       <c r="D13" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E13" t="n">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="F13" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G13" t="n">
         <v>0</v>
       </c>
       <c r="H13" t="n">
-        <v>26</v>
+        <v>41</v>
       </c>
       <c r="I13" t="n">
         <v>0</v>
@@ -6394,7 +6394,7 @@
         <v>0</v>
       </c>
       <c r="C14" t="n">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="D14" t="n">
         <v>1</v>
@@ -6409,7 +6409,7 @@
         <v>0</v>
       </c>
       <c r="H14" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="I14" t="n">
         <v>0</v>
@@ -6469,29 +6469,29 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>AREA_1422</t>
+          <t>413 - BAIRRO DA GRANJA - ESTRATO 2</t>
         </is>
       </c>
       <c r="B15" t="n">
         <v>0</v>
       </c>
       <c r="C15" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="D15" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="E15" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F15" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G15" t="n">
         <v>0</v>
       </c>
       <c r="H15" t="n">
-        <v>0</v>
+        <v>29</v>
       </c>
       <c r="I15" t="n">
         <v>0</v>
@@ -6558,22 +6558,22 @@
         <v>0</v>
       </c>
       <c r="C16" t="n">
-        <v>7</v>
+        <v>15</v>
       </c>
       <c r="D16" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="E16" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="F16" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="G16" t="n">
         <v>0</v>
       </c>
       <c r="H16" t="n">
-        <v>12</v>
+        <v>35</v>
       </c>
       <c r="I16" t="n">
         <v>0</v>
@@ -6715,29 +6715,29 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>AREA_1425</t>
+          <t>416 - CENTRO 2 - ESTRATO 2</t>
         </is>
       </c>
       <c r="B18" t="n">
         <v>0</v>
       </c>
       <c r="C18" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D18" t="n">
-        <v>0</v>
+        <v>18</v>
       </c>
       <c r="E18" t="n">
         <v>0</v>
       </c>
       <c r="F18" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G18" t="n">
         <v>0</v>
       </c>
       <c r="H18" t="n">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="I18" t="n">
         <v>0</v>
@@ -6797,29 +6797,29 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>AREA_1426</t>
+          <t>417 - CENTRO 3 - ESTRATO 2</t>
         </is>
       </c>
       <c r="B19" t="n">
         <v>0</v>
       </c>
       <c r="C19" t="n">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="D19" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="E19" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F19" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="G19" t="n">
         <v>0</v>
       </c>
       <c r="H19" t="n">
-        <v>0</v>
+        <v>23</v>
       </c>
       <c r="I19" t="n">
         <v>0</v>
@@ -6879,20 +6879,20 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>AREA_1427</t>
+          <t>418 - CENTRO 4 - ESTRATO 2</t>
         </is>
       </c>
       <c r="B20" t="n">
         <v>0</v>
       </c>
       <c r="C20" t="n">
-        <v>0</v>
+        <v>19</v>
       </c>
       <c r="D20" t="n">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="E20" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F20" t="n">
         <v>0</v>
@@ -6901,7 +6901,7 @@
         <v>0</v>
       </c>
       <c r="H20" t="n">
-        <v>0</v>
+        <v>32</v>
       </c>
       <c r="I20" t="n">
         <v>0</v>
@@ -6965,25 +6965,25 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C21" t="n">
+        <v>9</v>
+      </c>
+      <c r="D21" t="n">
         <v>5</v>
       </c>
-      <c r="D21" t="n">
-        <v>1</v>
-      </c>
       <c r="E21" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F21" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G21" t="n">
         <v>0</v>
       </c>
       <c r="H21" t="n">
-        <v>9</v>
+        <v>20</v>
       </c>
       <c r="I21" t="n">
         <v>0</v>
@@ -7047,16 +7047,16 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C22" t="n">
-        <v>16</v>
+        <v>27</v>
       </c>
       <c r="D22" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E22" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F22" t="n">
         <v>0</v>
@@ -7065,7 +7065,7 @@
         <v>0</v>
       </c>
       <c r="H22" t="n">
-        <v>20</v>
+        <v>35</v>
       </c>
       <c r="I22" t="n">
         <v>0</v>
@@ -7132,7 +7132,7 @@
         <v>0</v>
       </c>
       <c r="C23" t="n">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="D23" t="n">
         <v>2</v>
@@ -7141,13 +7141,13 @@
         <v>5</v>
       </c>
       <c r="F23" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G23" t="n">
         <v>0</v>
       </c>
       <c r="H23" t="n">
-        <v>26</v>
+        <v>33</v>
       </c>
       <c r="I23" t="n">
         <v>0</v>
@@ -7214,10 +7214,10 @@
         <v>0</v>
       </c>
       <c r="C24" t="n">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="D24" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E24" t="n">
         <v>3</v>
@@ -7229,7 +7229,7 @@
         <v>0</v>
       </c>
       <c r="H24" t="n">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="I24" t="n">
         <v>0</v>
@@ -7296,7 +7296,7 @@
         <v>1</v>
       </c>
       <c r="C25" t="n">
-        <v>11</v>
+        <v>24</v>
       </c>
       <c r="D25" t="n">
         <v>0</v>
@@ -7305,13 +7305,13 @@
         <v>1</v>
       </c>
       <c r="F25" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G25" t="n">
         <v>0</v>
       </c>
       <c r="H25" t="n">
-        <v>13</v>
+        <v>27</v>
       </c>
       <c r="I25" t="n">
         <v>0</v>
@@ -7375,16 +7375,16 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C26" t="n">
-        <v>11</v>
+        <v>22</v>
       </c>
       <c r="D26" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E26" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="F26" t="n">
         <v>1</v>
@@ -7393,7 +7393,7 @@
         <v>0</v>
       </c>
       <c r="H26" t="n">
-        <v>18</v>
+        <v>34</v>
       </c>
       <c r="I26" t="n">
         <v>0</v>
@@ -7621,17 +7621,17 @@
         </is>
       </c>
       <c r="B29" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C29" t="n">
+        <v>21</v>
+      </c>
+      <c r="D29" t="n">
+        <v>0</v>
+      </c>
+      <c r="E29" t="n">
         <v>15</v>
       </c>
-      <c r="D29" t="n">
-        <v>0</v>
-      </c>
-      <c r="E29" t="n">
-        <v>8</v>
-      </c>
       <c r="F29" t="n">
         <v>1</v>
       </c>
@@ -7639,7 +7639,7 @@
         <v>0</v>
       </c>
       <c r="H29" t="n">
-        <v>24</v>
+        <v>37</v>
       </c>
       <c r="I29" t="n">
         <v>0</v>
@@ -7706,22 +7706,22 @@
         <v>1</v>
       </c>
       <c r="C30" t="n">
-        <v>13</v>
+        <v>25</v>
       </c>
       <c r="D30" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E30" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="F30" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G30" t="n">
         <v>0</v>
       </c>
       <c r="H30" t="n">
-        <v>20</v>
+        <v>36</v>
       </c>
       <c r="I30" t="n">
         <v>0</v>
@@ -7785,25 +7785,25 @@
         </is>
       </c>
       <c r="B31" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C31" t="n">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="D31" t="n">
         <v>0</v>
       </c>
       <c r="E31" t="n">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="F31" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G31" t="n">
         <v>0</v>
       </c>
       <c r="H31" t="n">
-        <v>16</v>
+        <v>31</v>
       </c>
       <c r="I31" t="n">
         <v>0</v>
@@ -7870,13 +7870,13 @@
         <v>0</v>
       </c>
       <c r="C32" t="n">
-        <v>9</v>
+        <v>21</v>
       </c>
       <c r="D32" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E32" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="F32" t="n">
         <v>1</v>
@@ -7885,7 +7885,7 @@
         <v>0</v>
       </c>
       <c r="H32" t="n">
-        <v>17</v>
+        <v>32</v>
       </c>
       <c r="I32" t="n">
         <v>0</v>
@@ -7945,29 +7945,29 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>AREA_1450</t>
+          <t>431 - PANAMBI - ESTRATO 3</t>
         </is>
       </c>
       <c r="B33" t="n">
         <v>0</v>
       </c>
       <c r="C33" t="n">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="D33" t="n">
         <v>0</v>
       </c>
       <c r="E33" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F33" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G33" t="n">
         <v>0</v>
       </c>
       <c r="H33" t="n">
-        <v>0</v>
+        <v>18</v>
       </c>
       <c r="I33" t="n">
         <v>0</v>
@@ -8280,13 +8280,13 @@
         <v>0</v>
       </c>
       <c r="C37" t="n">
-        <v>10</v>
+        <v>22</v>
       </c>
       <c r="D37" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E37" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="F37" t="n">
         <v>0</v>
@@ -8295,7 +8295,7 @@
         <v>0</v>
       </c>
       <c r="H37" t="n">
-        <v>19</v>
+        <v>35</v>
       </c>
       <c r="I37" t="n">
         <v>0</v>
@@ -8526,13 +8526,13 @@
         <v>1</v>
       </c>
       <c r="C40" t="n">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="D40" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E40" t="n">
-        <v>8</v>
+        <v>17</v>
       </c>
       <c r="F40" t="n">
         <v>2</v>
@@ -8541,7 +8541,7 @@
         <v>0</v>
       </c>
       <c r="H40" t="n">
-        <v>25</v>
+        <v>42</v>
       </c>
       <c r="I40" t="n">
         <v>0</v>
@@ -8690,13 +8690,13 @@
         <v>0</v>
       </c>
       <c r="C42" t="n">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="D42" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E42" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="F42" t="n">
         <v>0</v>
@@ -8705,7 +8705,7 @@
         <v>0</v>
       </c>
       <c r="H42" t="n">
-        <v>18</v>
+        <v>36</v>
       </c>
       <c r="I42" t="n">
         <v>0</v>
@@ -8765,29 +8765,29 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>AREA_1485</t>
+          <t>440 - JARDIM IBIRAPUERA - ESTRATO 4</t>
         </is>
       </c>
       <c r="B43" t="n">
         <v>0</v>
       </c>
       <c r="C43" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="D43" t="n">
         <v>0</v>
       </c>
       <c r="E43" t="n">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="F43" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G43" t="n">
         <v>0</v>
       </c>
       <c r="H43" t="n">
-        <v>0</v>
+        <v>21</v>
       </c>
       <c r="I43" t="n">
         <v>0</v>
@@ -8847,29 +8847,29 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>AREA_1486</t>
+          <t>441 - PARQUE DOS IPES - ESTRATO 4</t>
         </is>
       </c>
       <c r="B44" t="n">
         <v>0</v>
       </c>
       <c r="C44" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="D44" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E44" t="n">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="F44" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G44" t="n">
         <v>0</v>
       </c>
       <c r="H44" t="n">
-        <v>0</v>
+        <v>26</v>
       </c>
       <c r="I44" t="n">
         <v>0</v>
@@ -8933,10 +8933,10 @@
         </is>
       </c>
       <c r="B45" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C45" t="n">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="D45" t="n">
         <v>0</v>
@@ -8951,7 +8951,7 @@
         <v>0</v>
       </c>
       <c r="H45" t="n">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="I45" t="n">
         <v>0</v>
@@ -9011,29 +9011,29 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>AREA_2596</t>
+          <t>446 - GUY VILELA - ESTRATO 4</t>
         </is>
       </c>
       <c r="B46" t="n">
         <v>0</v>
       </c>
       <c r="C46" t="n">
-        <v>0</v>
+        <v>21</v>
       </c>
       <c r="D46" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="E46" t="n">
-        <v>0</v>
+        <v>18</v>
       </c>
       <c r="F46" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="G46" t="n">
         <v>0</v>
       </c>
       <c r="H46" t="n">
-        <v>0</v>
+        <v>48</v>
       </c>
       <c r="I46" t="n">
         <v>0</v>
@@ -9182,13 +9182,13 @@
         <v>0</v>
       </c>
       <c r="C48" t="n">
-        <v>13</v>
+        <v>25</v>
       </c>
       <c r="D48" t="n">
         <v>0</v>
       </c>
       <c r="E48" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="F48" t="n">
         <v>1</v>
@@ -9197,7 +9197,7 @@
         <v>0</v>
       </c>
       <c r="H48" t="n">
-        <v>15</v>
+        <v>32</v>
       </c>
       <c r="I48" t="n">
         <v>0</v>
@@ -9343,25 +9343,25 @@
         </is>
       </c>
       <c r="B50" t="n">
-        <v>23</v>
+        <v>30</v>
       </c>
       <c r="C50" t="n">
-        <v>449</v>
+        <v>770</v>
       </c>
       <c r="D50" t="n">
-        <v>44</v>
+        <v>118</v>
       </c>
       <c r="E50" t="n">
-        <v>216</v>
+        <v>349</v>
       </c>
       <c r="F50" t="n">
-        <v>39</v>
+        <v>81</v>
       </c>
       <c r="G50" t="n">
         <v>0</v>
       </c>
       <c r="H50" t="n">
-        <v>748</v>
+        <v>1318</v>
       </c>
       <c r="I50" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Atualização automática LIRAa 2026-08-05 11:15 UTC
</commit_message>
<xml_diff>
--- a/data/LIRA_COMPLETO_latest.xlsx
+++ b/data/LIRA_COMPLETO_latest.xlsx
@@ -555,29 +555,29 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>AREA_1236</t>
+          <t>400 - JULIA CARDINAL - ESTRATO 1</t>
         </is>
       </c>
       <c r="B2" t="n">
         <v>0</v>
       </c>
       <c r="C2" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="D2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E2" t="n">
-        <v>0</v>
+        <v>19</v>
       </c>
       <c r="F2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G2" t="n">
         <v>0</v>
       </c>
       <c r="H2" t="n">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="I2" t="n">
         <v>0</v>
@@ -969,10 +969,10 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C7" t="n">
-        <v>9</v>
+        <v>21</v>
       </c>
       <c r="D7" t="n">
         <v>1</v>
@@ -987,7 +987,7 @@
         <v>0</v>
       </c>
       <c r="H7" t="n">
-        <v>13</v>
+        <v>25</v>
       </c>
       <c r="I7" t="n">
         <v>0</v>
@@ -1543,25 +1543,25 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C14" t="n">
-        <v>165</v>
+        <v>184</v>
       </c>
       <c r="D14" t="n">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="E14" t="n">
-        <v>100</v>
+        <v>119</v>
       </c>
       <c r="F14" t="n">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="G14" t="n">
         <v>0</v>
       </c>
       <c r="H14" t="n">
-        <v>313</v>
+        <v>355</v>
       </c>
       <c r="I14" t="n">
         <v>0</v>
@@ -4198,22 +4198,22 @@
         <v>1</v>
       </c>
       <c r="C2" t="n">
-        <v>14</v>
+        <v>29</v>
       </c>
       <c r="D2" t="n">
+        <v>7</v>
+      </c>
+      <c r="E2" t="n">
+        <v>8</v>
+      </c>
+      <c r="F2" t="n">
         <v>2</v>
       </c>
-      <c r="E2" t="n">
-        <v>3</v>
-      </c>
-      <c r="F2" t="n">
-        <v>0</v>
-      </c>
       <c r="G2" t="n">
         <v>0</v>
       </c>
       <c r="H2" t="n">
-        <v>19</v>
+        <v>46</v>
       </c>
       <c r="I2" t="n">
         <v>0</v>
@@ -4444,13 +4444,13 @@
         <v>1</v>
       </c>
       <c r="C5" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="D5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E5" t="n">
-        <v>7</v>
+        <v>16</v>
       </c>
       <c r="F5" t="n">
         <v>2</v>
@@ -4459,7 +4459,7 @@
         <v>0</v>
       </c>
       <c r="H5" t="n">
-        <v>20</v>
+        <v>34</v>
       </c>
       <c r="I5" t="n">
         <v>0</v>
@@ -5182,22 +5182,22 @@
         <v>5</v>
       </c>
       <c r="C14" t="n">
-        <v>180</v>
+        <v>199</v>
       </c>
       <c r="D14" t="n">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="E14" t="n">
-        <v>115</v>
+        <v>129</v>
       </c>
       <c r="F14" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="G14" t="n">
         <v>0</v>
       </c>
       <c r="H14" t="n">
-        <v>329</v>
+        <v>370</v>
       </c>
       <c r="I14" t="n">
         <v>0</v>
@@ -5403,29 +5403,29 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>AREA_1236</t>
+          <t>400 - JULIA CARDINAL - ESTRATO 1</t>
         </is>
       </c>
       <c r="B2" t="n">
         <v>0</v>
       </c>
       <c r="C2" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="D2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E2" t="n">
-        <v>0</v>
+        <v>19</v>
       </c>
       <c r="F2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G2" t="n">
         <v>0</v>
       </c>
       <c r="H2" t="n">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="I2" t="n">
         <v>0</v>
@@ -5817,10 +5817,10 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C7" t="n">
-        <v>9</v>
+        <v>21</v>
       </c>
       <c r="D7" t="n">
         <v>1</v>
@@ -5835,7 +5835,7 @@
         <v>0</v>
       </c>
       <c r="H7" t="n">
-        <v>13</v>
+        <v>25</v>
       </c>
       <c r="I7" t="n">
         <v>0</v>
@@ -8362,22 +8362,22 @@
         <v>1</v>
       </c>
       <c r="C38" t="n">
-        <v>14</v>
+        <v>29</v>
       </c>
       <c r="D38" t="n">
+        <v>7</v>
+      </c>
+      <c r="E38" t="n">
+        <v>8</v>
+      </c>
+      <c r="F38" t="n">
         <v>2</v>
       </c>
-      <c r="E38" t="n">
-        <v>3</v>
-      </c>
-      <c r="F38" t="n">
-        <v>0</v>
-      </c>
       <c r="G38" t="n">
         <v>0</v>
       </c>
       <c r="H38" t="n">
-        <v>19</v>
+        <v>46</v>
       </c>
       <c r="I38" t="n">
         <v>0</v>
@@ -8608,13 +8608,13 @@
         <v>1</v>
       </c>
       <c r="C41" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="D41" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E41" t="n">
-        <v>7</v>
+        <v>16</v>
       </c>
       <c r="F41" t="n">
         <v>2</v>
@@ -8623,7 +8623,7 @@
         <v>0</v>
       </c>
       <c r="H41" t="n">
-        <v>20</v>
+        <v>34</v>
       </c>
       <c r="I41" t="n">
         <v>0</v>
@@ -9343,25 +9343,25 @@
         </is>
       </c>
       <c r="B50" t="n">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="C50" t="n">
-        <v>770</v>
+        <v>808</v>
       </c>
       <c r="D50" t="n">
-        <v>118</v>
+        <v>126</v>
       </c>
       <c r="E50" t="n">
-        <v>349</v>
+        <v>382</v>
       </c>
       <c r="F50" t="n">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="G50" t="n">
         <v>0</v>
       </c>
       <c r="H50" t="n">
-        <v>1318</v>
+        <v>1401</v>
       </c>
       <c r="I50" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Atualização automática LIRAa 2026-08-05 13:45 UTC
</commit_message>
<xml_diff>
--- a/data/LIRA_COMPLETO_latest.xlsx
+++ b/data/LIRA_COMPLETO_latest.xlsx
@@ -726,13 +726,13 @@
         <v>0</v>
       </c>
       <c r="C4" t="n">
-        <v>11</v>
+        <v>23</v>
       </c>
       <c r="D4" t="n">
         <v>0</v>
       </c>
       <c r="E4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F4" t="n">
         <v>0</v>
@@ -741,7 +741,7 @@
         <v>0</v>
       </c>
       <c r="H4" t="n">
-        <v>15</v>
+        <v>28</v>
       </c>
       <c r="I4" t="n">
         <v>0</v>
@@ -1546,13 +1546,13 @@
         <v>6</v>
       </c>
       <c r="C14" t="n">
-        <v>184</v>
+        <v>196</v>
       </c>
       <c r="D14" t="n">
         <v>28</v>
       </c>
       <c r="E14" t="n">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="F14" t="n">
         <v>24</v>
@@ -1561,7 +1561,7 @@
         <v>0</v>
       </c>
       <c r="H14" t="n">
-        <v>355</v>
+        <v>368</v>
       </c>
       <c r="I14" t="n">
         <v>0</v>
@@ -1774,10 +1774,10 @@
         <v>0</v>
       </c>
       <c r="C2" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E2" t="n">
         <v>3</v>
@@ -1859,10 +1859,10 @@
         <v>20</v>
       </c>
       <c r="D3" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F3" t="n">
         <v>3</v>
@@ -2430,16 +2430,16 @@
         <v>4</v>
       </c>
       <c r="C10" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="D10" t="n">
         <v>4</v>
       </c>
       <c r="E10" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F10" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G10" t="n">
         <v>0</v>
@@ -2512,13 +2512,13 @@
         <v>0</v>
       </c>
       <c r="C11" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D11" t="n">
         <v>2</v>
       </c>
       <c r="E11" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F11" t="n">
         <v>3</v>
@@ -2676,16 +2676,16 @@
         <v>6</v>
       </c>
       <c r="C13" t="n">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="D13" t="n">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="E13" t="n">
         <v>31</v>
       </c>
       <c r="F13" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="G13" t="n">
         <v>0</v>
@@ -3068,13 +3068,13 @@
         <v>0</v>
       </c>
       <c r="C4" t="n">
-        <v>17</v>
+        <v>26</v>
       </c>
       <c r="D4" t="n">
         <v>0</v>
       </c>
       <c r="E4" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="F4" t="n">
         <v>3</v>
@@ -3083,7 +3083,7 @@
         <v>0</v>
       </c>
       <c r="H4" t="n">
-        <v>25</v>
+        <v>38</v>
       </c>
       <c r="I4" t="n">
         <v>0</v>
@@ -3150,13 +3150,13 @@
         <v>1</v>
       </c>
       <c r="C5" t="n">
+        <v>23</v>
+      </c>
+      <c r="D5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E5" t="n">
         <v>21</v>
-      </c>
-      <c r="D5" t="n">
-        <v>1</v>
-      </c>
-      <c r="E5" t="n">
-        <v>19</v>
       </c>
       <c r="F5" t="n">
         <v>2</v>
@@ -3165,7 +3165,7 @@
         <v>0</v>
       </c>
       <c r="H5" t="n">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="I5" t="n">
         <v>0</v>
@@ -3970,13 +3970,13 @@
         <v>15</v>
       </c>
       <c r="C15" t="n">
-        <v>259</v>
+        <v>270</v>
       </c>
       <c r="D15" t="n">
         <v>16</v>
       </c>
       <c r="E15" t="n">
-        <v>103</v>
+        <v>109</v>
       </c>
       <c r="F15" t="n">
         <v>18</v>
@@ -3985,7 +3985,7 @@
         <v>0</v>
       </c>
       <c r="H15" t="n">
-        <v>396</v>
+        <v>413</v>
       </c>
       <c r="I15" t="n">
         <v>0</v>
@@ -4280,13 +4280,13 @@
         <v>0</v>
       </c>
       <c r="C3" t="n">
-        <v>7</v>
+        <v>15</v>
       </c>
       <c r="D3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E3" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="F3" t="n">
         <v>0</v>
@@ -4295,7 +4295,7 @@
         <v>0</v>
       </c>
       <c r="H3" t="n">
-        <v>11</v>
+        <v>25</v>
       </c>
       <c r="I3" t="n">
         <v>0</v>
@@ -4362,13 +4362,13 @@
         <v>1</v>
       </c>
       <c r="C4" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D4" t="n">
         <v>2</v>
       </c>
       <c r="E4" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="F4" t="n">
         <v>2</v>
@@ -5182,13 +5182,13 @@
         <v>5</v>
       </c>
       <c r="C14" t="n">
-        <v>199</v>
+        <v>206</v>
       </c>
       <c r="D14" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="E14" t="n">
-        <v>129</v>
+        <v>135</v>
       </c>
       <c r="F14" t="n">
         <v>22</v>
@@ -5197,7 +5197,7 @@
         <v>0</v>
       </c>
       <c r="H14" t="n">
-        <v>370</v>
+        <v>384</v>
       </c>
       <c r="I14" t="n">
         <v>0</v>
@@ -5574,13 +5574,13 @@
         <v>0</v>
       </c>
       <c r="C4" t="n">
-        <v>11</v>
+        <v>23</v>
       </c>
       <c r="D4" t="n">
         <v>0</v>
       </c>
       <c r="E4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F4" t="n">
         <v>0</v>
@@ -5589,7 +5589,7 @@
         <v>0</v>
       </c>
       <c r="H4" t="n">
-        <v>15</v>
+        <v>28</v>
       </c>
       <c r="I4" t="n">
         <v>0</v>
@@ -6394,10 +6394,10 @@
         <v>0</v>
       </c>
       <c r="C14" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D14" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E14" t="n">
         <v>3</v>
@@ -6479,10 +6479,10 @@
         <v>20</v>
       </c>
       <c r="D15" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F15" t="n">
         <v>3</v>
@@ -7050,16 +7050,16 @@
         <v>4</v>
       </c>
       <c r="C22" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="D22" t="n">
         <v>4</v>
       </c>
       <c r="E22" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F22" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G22" t="n">
         <v>0</v>
@@ -7132,13 +7132,13 @@
         <v>0</v>
       </c>
       <c r="C23" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D23" t="n">
         <v>2</v>
       </c>
       <c r="E23" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F23" t="n">
         <v>3</v>
@@ -7460,13 +7460,13 @@
         <v>0</v>
       </c>
       <c r="C27" t="n">
-        <v>17</v>
+        <v>26</v>
       </c>
       <c r="D27" t="n">
         <v>0</v>
       </c>
       <c r="E27" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="F27" t="n">
         <v>3</v>
@@ -7475,7 +7475,7 @@
         <v>0</v>
       </c>
       <c r="H27" t="n">
-        <v>25</v>
+        <v>38</v>
       </c>
       <c r="I27" t="n">
         <v>0</v>
@@ -7542,13 +7542,13 @@
         <v>1</v>
       </c>
       <c r="C28" t="n">
+        <v>23</v>
+      </c>
+      <c r="D28" t="n">
+        <v>1</v>
+      </c>
+      <c r="E28" t="n">
         <v>21</v>
-      </c>
-      <c r="D28" t="n">
-        <v>1</v>
-      </c>
-      <c r="E28" t="n">
-        <v>19</v>
       </c>
       <c r="F28" t="n">
         <v>2</v>
@@ -7557,7 +7557,7 @@
         <v>0</v>
       </c>
       <c r="H28" t="n">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="I28" t="n">
         <v>0</v>
@@ -8444,13 +8444,13 @@
         <v>0</v>
       </c>
       <c r="C39" t="n">
-        <v>7</v>
+        <v>15</v>
       </c>
       <c r="D39" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E39" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="F39" t="n">
         <v>0</v>
@@ -8459,7 +8459,7 @@
         <v>0</v>
       </c>
       <c r="H39" t="n">
-        <v>11</v>
+        <v>25</v>
       </c>
       <c r="I39" t="n">
         <v>0</v>
@@ -8526,13 +8526,13 @@
         <v>1</v>
       </c>
       <c r="C40" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D40" t="n">
         <v>2</v>
       </c>
       <c r="E40" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="F40" t="n">
         <v>2</v>
@@ -9346,22 +9346,22 @@
         <v>32</v>
       </c>
       <c r="C50" t="n">
-        <v>808</v>
+        <v>839</v>
       </c>
       <c r="D50" t="n">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="E50" t="n">
-        <v>382</v>
+        <v>395</v>
       </c>
       <c r="F50" t="n">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="G50" t="n">
         <v>0</v>
       </c>
       <c r="H50" t="n">
-        <v>1401</v>
+        <v>1445</v>
       </c>
       <c r="I50" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Atualização automática LIRAa 2026-08-05 15:34 UTC
</commit_message>
<xml_diff>
--- a/data/LIRA_COMPLETO_latest.xlsx
+++ b/data/LIRA_COMPLETO_latest.xlsx
@@ -996,7 +996,7 @@
         <v>0</v>
       </c>
       <c r="K7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L7" t="n">
         <v>0</v>
@@ -1011,10 +1011,10 @@
         <v>0</v>
       </c>
       <c r="P7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R7" t="n">
         <v>0</v>
@@ -1026,7 +1026,7 @@
         <v>0</v>
       </c>
       <c r="U7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V7" t="n">
         <v>0</v>
@@ -1570,7 +1570,7 @@
         <v>1</v>
       </c>
       <c r="K14" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L14" t="n">
         <v>0</v>
@@ -1585,10 +1585,10 @@
         <v>0</v>
       </c>
       <c r="P14" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="Q14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R14" t="n">
         <v>0</v>
@@ -1600,7 +1600,7 @@
         <v>0</v>
       </c>
       <c r="U14" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="V14" t="n">
         <v>0</v>
@@ -2454,7 +2454,7 @@
         <v>1</v>
       </c>
       <c r="K10" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="L10" t="n">
         <v>0</v>
@@ -2469,10 +2469,10 @@
         <v>0</v>
       </c>
       <c r="P10" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="Q10" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="R10" t="n">
         <v>0</v>
@@ -2484,7 +2484,7 @@
         <v>0</v>
       </c>
       <c r="U10" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="V10" t="n">
         <v>0</v>
@@ -2700,7 +2700,7 @@
         <v>1</v>
       </c>
       <c r="K13" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="L13" t="n">
         <v>0</v>
@@ -2715,10 +2715,10 @@
         <v>0</v>
       </c>
       <c r="P13" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="Q13" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="R13" t="n">
         <v>0</v>
@@ -2730,7 +2730,7 @@
         <v>0</v>
       </c>
       <c r="U13" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="V13" t="n">
         <v>0</v>
@@ -3177,7 +3177,7 @@
         <v>0</v>
       </c>
       <c r="L5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M5" t="n">
         <v>0</v>
@@ -3189,10 +3189,10 @@
         <v>0</v>
       </c>
       <c r="P5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R5" t="n">
         <v>0</v>
@@ -3204,7 +3204,7 @@
         <v>0</v>
       </c>
       <c r="U5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V5" t="n">
         <v>0</v>
@@ -3475,16 +3475,16 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C9" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D9" t="n">
         <v>3</v>
       </c>
       <c r="E9" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="F9" t="n">
         <v>1</v>
@@ -3493,7 +3493,7 @@
         <v>0</v>
       </c>
       <c r="H9" t="n">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="I9" t="n">
         <v>0</v>
@@ -3663,10 +3663,10 @@
         <v>0</v>
       </c>
       <c r="J11" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L11" t="n">
         <v>0</v>
@@ -3675,16 +3675,16 @@
         <v>0</v>
       </c>
       <c r="N11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O11" t="n">
         <v>0</v>
       </c>
       <c r="P11" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="Q11" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="R11" t="n">
         <v>0</v>
@@ -3696,10 +3696,10 @@
         <v>0</v>
       </c>
       <c r="U11" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="V11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="W11" t="n">
         <v>0</v>
@@ -3711,7 +3711,7 @@
         <v>0</v>
       </c>
       <c r="Z11" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="12">
@@ -3967,16 +3967,16 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="C15" t="n">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="D15" t="n">
         <v>16</v>
       </c>
       <c r="E15" t="n">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="F15" t="n">
         <v>18</v>
@@ -3985,34 +3985,34 @@
         <v>0</v>
       </c>
       <c r="H15" t="n">
-        <v>413</v>
+        <v>417</v>
       </c>
       <c r="I15" t="n">
         <v>0</v>
       </c>
       <c r="J15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K15" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L15" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M15" t="n">
         <v>0</v>
       </c>
       <c r="N15" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O15" t="n">
         <v>0</v>
       </c>
       <c r="P15" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="Q15" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="R15" t="n">
         <v>0</v>
@@ -4024,10 +4024,10 @@
         <v>0</v>
       </c>
       <c r="U15" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="V15" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="W15" t="n">
         <v>0</v>
@@ -4039,7 +4039,7 @@
         <v>0</v>
       </c>
       <c r="Z15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
   </sheetData>
@@ -4805,28 +4805,28 @@
         <v>0</v>
       </c>
       <c r="N9" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="O9" t="n">
         <v>0</v>
       </c>
       <c r="P9" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="Q9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R9" t="n">
         <v>0</v>
       </c>
       <c r="S9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T9" t="n">
         <v>0</v>
       </c>
       <c r="U9" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="V9" t="n">
         <v>0</v>
@@ -5215,28 +5215,28 @@
         <v>0</v>
       </c>
       <c r="N14" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="O14" t="n">
         <v>0</v>
       </c>
       <c r="P14" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="Q14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R14" t="n">
         <v>0</v>
       </c>
       <c r="S14" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="T14" t="n">
         <v>0</v>
       </c>
       <c r="U14" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="V14" t="n">
         <v>0</v>
@@ -5844,7 +5844,7 @@
         <v>0</v>
       </c>
       <c r="K7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L7" t="n">
         <v>0</v>
@@ -5859,10 +5859,10 @@
         <v>0</v>
       </c>
       <c r="P7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R7" t="n">
         <v>0</v>
@@ -5874,7 +5874,7 @@
         <v>0</v>
       </c>
       <c r="U7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V7" t="n">
         <v>0</v>
@@ -7074,7 +7074,7 @@
         <v>1</v>
       </c>
       <c r="K22" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="L22" t="n">
         <v>0</v>
@@ -7089,10 +7089,10 @@
         <v>0</v>
       </c>
       <c r="P22" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="Q22" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="R22" t="n">
         <v>0</v>
@@ -7104,7 +7104,7 @@
         <v>0</v>
       </c>
       <c r="U22" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="V22" t="n">
         <v>0</v>
@@ -7569,7 +7569,7 @@
         <v>0</v>
       </c>
       <c r="L28" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M28" t="n">
         <v>0</v>
@@ -7581,10 +7581,10 @@
         <v>0</v>
       </c>
       <c r="P28" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q28" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R28" t="n">
         <v>0</v>
@@ -7596,7 +7596,7 @@
         <v>0</v>
       </c>
       <c r="U28" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V28" t="n">
         <v>0</v>
@@ -7867,16 +7867,16 @@
         </is>
       </c>
       <c r="B32" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C32" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D32" t="n">
         <v>3</v>
       </c>
       <c r="E32" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="F32" t="n">
         <v>1</v>
@@ -7885,7 +7885,7 @@
         <v>0</v>
       </c>
       <c r="H32" t="n">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="I32" t="n">
         <v>0</v>
@@ -8055,10 +8055,10 @@
         <v>0</v>
       </c>
       <c r="J34" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K34" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L34" t="n">
         <v>0</v>
@@ -8067,16 +8067,16 @@
         <v>0</v>
       </c>
       <c r="N34" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O34" t="n">
         <v>0</v>
       </c>
       <c r="P34" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="Q34" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="R34" t="n">
         <v>0</v>
@@ -8088,10 +8088,10 @@
         <v>0</v>
       </c>
       <c r="U34" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="V34" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="W34" t="n">
         <v>0</v>
@@ -8103,7 +8103,7 @@
         <v>0</v>
       </c>
       <c r="Z34" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="35">
@@ -8969,28 +8969,28 @@
         <v>0</v>
       </c>
       <c r="N45" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="O45" t="n">
         <v>0</v>
       </c>
       <c r="P45" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="Q45" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R45" t="n">
         <v>0</v>
       </c>
       <c r="S45" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T45" t="n">
         <v>0</v>
       </c>
       <c r="U45" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="V45" t="n">
         <v>0</v>
@@ -9343,16 +9343,16 @@
         </is>
       </c>
       <c r="B50" t="n">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C50" t="n">
-        <v>839</v>
+        <v>840</v>
       </c>
       <c r="D50" t="n">
         <v>125</v>
       </c>
       <c r="E50" t="n">
-        <v>395</v>
+        <v>398</v>
       </c>
       <c r="F50" t="n">
         <v>86</v>
@@ -9361,61 +9361,61 @@
         <v>0</v>
       </c>
       <c r="H50" t="n">
-        <v>1445</v>
+        <v>1449</v>
       </c>
       <c r="I50" t="n">
         <v>0</v>
       </c>
       <c r="J50" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K50" t="n">
+        <v>6</v>
+      </c>
+      <c r="L50" t="n">
+        <v>1</v>
+      </c>
+      <c r="M50" t="n">
+        <v>0</v>
+      </c>
+      <c r="N50" t="n">
+        <v>4</v>
+      </c>
+      <c r="O50" t="n">
+        <v>0</v>
+      </c>
+      <c r="P50" t="n">
+        <v>15</v>
+      </c>
+      <c r="Q50" t="n">
+        <v>11</v>
+      </c>
+      <c r="R50" t="n">
+        <v>0</v>
+      </c>
+      <c r="S50" t="n">
+        <v>4</v>
+      </c>
+      <c r="T50" t="n">
+        <v>0</v>
+      </c>
+      <c r="U50" t="n">
+        <v>15</v>
+      </c>
+      <c r="V50" t="n">
+        <v>1</v>
+      </c>
+      <c r="W50" t="n">
+        <v>0</v>
+      </c>
+      <c r="X50" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y50" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z50" t="n">
         <v>2</v>
-      </c>
-      <c r="L50" t="n">
-        <v>0</v>
-      </c>
-      <c r="M50" t="n">
-        <v>0</v>
-      </c>
-      <c r="N50" t="n">
-        <v>1</v>
-      </c>
-      <c r="O50" t="n">
-        <v>0</v>
-      </c>
-      <c r="P50" t="n">
-        <v>6</v>
-      </c>
-      <c r="Q50" t="n">
-        <v>3</v>
-      </c>
-      <c r="R50" t="n">
-        <v>0</v>
-      </c>
-      <c r="S50" t="n">
-        <v>3</v>
-      </c>
-      <c r="T50" t="n">
-        <v>0</v>
-      </c>
-      <c r="U50" t="n">
-        <v>6</v>
-      </c>
-      <c r="V50" t="n">
-        <v>0</v>
-      </c>
-      <c r="W50" t="n">
-        <v>0</v>
-      </c>
-      <c r="X50" t="n">
-        <v>1</v>
-      </c>
-      <c r="Y50" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z50" t="n">
-        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualização automática LIRAa 2026-08-05 17:31 UTC
</commit_message>
<xml_diff>
--- a/data/LIRA_COMPLETO_latest.xlsx
+++ b/data/LIRA_COMPLETO_latest.xlsx
@@ -3402,7 +3402,7 @@
         <v>0</v>
       </c>
       <c r="E8" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="F8" t="n">
         <v>3</v>
@@ -3411,7 +3411,7 @@
         <v>0</v>
       </c>
       <c r="H8" t="n">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="I8" t="n">
         <v>0</v>
@@ -3976,7 +3976,7 @@
         <v>16</v>
       </c>
       <c r="E15" t="n">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="F15" t="n">
         <v>18</v>
@@ -3985,7 +3985,7 @@
         <v>0</v>
       </c>
       <c r="H15" t="n">
-        <v>417</v>
+        <v>420</v>
       </c>
       <c r="I15" t="n">
         <v>0</v>
@@ -7794,7 +7794,7 @@
         <v>0</v>
       </c>
       <c r="E31" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="F31" t="n">
         <v>3</v>
@@ -7803,7 +7803,7 @@
         <v>0</v>
       </c>
       <c r="H31" t="n">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="I31" t="n">
         <v>0</v>
@@ -9352,7 +9352,7 @@
         <v>125</v>
       </c>
       <c r="E50" t="n">
-        <v>398</v>
+        <v>401</v>
       </c>
       <c r="F50" t="n">
         <v>86</v>
@@ -9361,7 +9361,7 @@
         <v>0</v>
       </c>
       <c r="H50" t="n">
-        <v>1449</v>
+        <v>1452</v>
       </c>
       <c r="I50" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Atualização automática LIRAa 2026-08-05 20:26 UTC
</commit_message>
<xml_diff>
--- a/data/LIRA_COMPLETO_latest.xlsx
+++ b/data/LIRA_COMPLETO_latest.xlsx
@@ -4277,10 +4277,10 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C3" t="n">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="D3" t="n">
         <v>2</v>
@@ -4295,7 +4295,7 @@
         <v>0</v>
       </c>
       <c r="H3" t="n">
-        <v>25</v>
+        <v>32</v>
       </c>
       <c r="I3" t="n">
         <v>0</v>
@@ -4936,13 +4936,13 @@
         <v>0</v>
       </c>
       <c r="C11" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="D11" t="n">
         <v>0</v>
       </c>
       <c r="E11" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="F11" t="n">
         <v>1</v>
@@ -4951,7 +4951,7 @@
         <v>0</v>
       </c>
       <c r="H11" t="n">
-        <v>9</v>
+        <v>16</v>
       </c>
       <c r="I11" t="n">
         <v>0</v>
@@ -5179,16 +5179,16 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C14" t="n">
-        <v>206</v>
+        <v>217</v>
       </c>
       <c r="D14" t="n">
         <v>21</v>
       </c>
       <c r="E14" t="n">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="F14" t="n">
         <v>22</v>
@@ -5197,7 +5197,7 @@
         <v>0</v>
       </c>
       <c r="H14" t="n">
-        <v>384</v>
+        <v>398</v>
       </c>
       <c r="I14" t="n">
         <v>0</v>
@@ -8441,10 +8441,10 @@
         </is>
       </c>
       <c r="B39" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C39" t="n">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="D39" t="n">
         <v>2</v>
@@ -8459,7 +8459,7 @@
         <v>0</v>
       </c>
       <c r="H39" t="n">
-        <v>25</v>
+        <v>32</v>
       </c>
       <c r="I39" t="n">
         <v>0</v>
@@ -9100,13 +9100,13 @@
         <v>0</v>
       </c>
       <c r="C47" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="D47" t="n">
         <v>0</v>
       </c>
       <c r="E47" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="F47" t="n">
         <v>1</v>
@@ -9115,7 +9115,7 @@
         <v>0</v>
       </c>
       <c r="H47" t="n">
-        <v>9</v>
+        <v>16</v>
       </c>
       <c r="I47" t="n">
         <v>0</v>
@@ -9343,16 +9343,16 @@
         </is>
       </c>
       <c r="B50" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C50" t="n">
-        <v>840</v>
+        <v>851</v>
       </c>
       <c r="D50" t="n">
         <v>125</v>
       </c>
       <c r="E50" t="n">
-        <v>401</v>
+        <v>404</v>
       </c>
       <c r="F50" t="n">
         <v>86</v>
@@ -9361,7 +9361,7 @@
         <v>0</v>
       </c>
       <c r="H50" t="n">
-        <v>1452</v>
+        <v>1466</v>
       </c>
       <c r="I50" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Atualização automática LIRAa 2026-08-05 23:08 UTC
</commit_message>
<xml_diff>
--- a/data/LIRA_COMPLETO_latest.xlsx
+++ b/data/LIRA_COMPLETO_latest.xlsx
@@ -723,10 +723,10 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C4" t="n">
-        <v>23</v>
+        <v>30</v>
       </c>
       <c r="D4" t="n">
         <v>0</v>
@@ -735,13 +735,13 @@
         <v>5</v>
       </c>
       <c r="F4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G4" t="n">
         <v>0</v>
       </c>
       <c r="H4" t="n">
-        <v>28</v>
+        <v>36</v>
       </c>
       <c r="I4" t="n">
         <v>0</v>
@@ -1543,10 +1543,10 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C14" t="n">
-        <v>196</v>
+        <v>203</v>
       </c>
       <c r="D14" t="n">
         <v>28</v>
@@ -1555,13 +1555,13 @@
         <v>120</v>
       </c>
       <c r="F14" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="G14" t="n">
         <v>0</v>
       </c>
       <c r="H14" t="n">
-        <v>368</v>
+        <v>376</v>
       </c>
       <c r="I14" t="n">
         <v>0</v>
@@ -2269,10 +2269,10 @@
         <v>19</v>
       </c>
       <c r="D8" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E8" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F8" t="n">
         <v>0</v>
@@ -2281,7 +2281,7 @@
         <v>0</v>
       </c>
       <c r="H8" t="n">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="I8" t="n">
         <v>0</v>
@@ -2348,22 +2348,22 @@
         <v>2</v>
       </c>
       <c r="C9" t="n">
-        <v>9</v>
+        <v>16</v>
       </c>
       <c r="D9" t="n">
+        <v>11</v>
+      </c>
+      <c r="E9" t="n">
         <v>5</v>
       </c>
-      <c r="E9" t="n">
-        <v>4</v>
-      </c>
       <c r="F9" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G9" t="n">
         <v>0</v>
       </c>
       <c r="H9" t="n">
-        <v>20</v>
+        <v>35</v>
       </c>
       <c r="I9" t="n">
         <v>0</v>
@@ -2676,22 +2676,22 @@
         <v>6</v>
       </c>
       <c r="C13" t="n">
-        <v>167</v>
+        <v>174</v>
       </c>
       <c r="D13" t="n">
-        <v>60</v>
+        <v>67</v>
       </c>
       <c r="E13" t="n">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="F13" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="G13" t="n">
         <v>0</v>
       </c>
       <c r="H13" t="n">
-        <v>280</v>
+        <v>297</v>
       </c>
       <c r="I13" t="n">
         <v>0</v>
@@ -3560,22 +3560,22 @@
         <v>0</v>
       </c>
       <c r="C10" t="n">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="D10" t="n">
         <v>0</v>
       </c>
       <c r="E10" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="F10" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G10" t="n">
         <v>0</v>
       </c>
       <c r="H10" t="n">
-        <v>18</v>
+        <v>30</v>
       </c>
       <c r="I10" t="n">
         <v>0</v>
@@ -3724,13 +3724,13 @@
         <v>0</v>
       </c>
       <c r="C12" t="n">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="D12" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E12" t="n">
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="F12" t="n">
         <v>0</v>
@@ -3739,7 +3739,7 @@
         <v>0</v>
       </c>
       <c r="H12" t="n">
-        <v>11</v>
+        <v>27</v>
       </c>
       <c r="I12" t="n">
         <v>0</v>
@@ -3970,22 +3970,22 @@
         <v>17</v>
       </c>
       <c r="C15" t="n">
-        <v>271</v>
+        <v>285</v>
       </c>
       <c r="D15" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="E15" t="n">
-        <v>115</v>
+        <v>126</v>
       </c>
       <c r="F15" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="G15" t="n">
         <v>0</v>
       </c>
       <c r="H15" t="n">
-        <v>420</v>
+        <v>448</v>
       </c>
       <c r="I15" t="n">
         <v>0</v>
@@ -4608,22 +4608,22 @@
         <v>0</v>
       </c>
       <c r="C7" t="n">
-        <v>7</v>
+        <v>20</v>
       </c>
       <c r="D7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E7" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="F7" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G7" t="n">
         <v>0</v>
       </c>
       <c r="H7" t="n">
-        <v>21</v>
+        <v>38</v>
       </c>
       <c r="I7" t="n">
         <v>0</v>
@@ -5182,22 +5182,22 @@
         <v>6</v>
       </c>
       <c r="C14" t="n">
-        <v>217</v>
+        <v>230</v>
       </c>
       <c r="D14" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E14" t="n">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="F14" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="G14" t="n">
         <v>0</v>
       </c>
       <c r="H14" t="n">
-        <v>398</v>
+        <v>415</v>
       </c>
       <c r="I14" t="n">
         <v>0</v>
@@ -5571,10 +5571,10 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C4" t="n">
-        <v>23</v>
+        <v>30</v>
       </c>
       <c r="D4" t="n">
         <v>0</v>
@@ -5583,13 +5583,13 @@
         <v>5</v>
       </c>
       <c r="F4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G4" t="n">
         <v>0</v>
       </c>
       <c r="H4" t="n">
-        <v>28</v>
+        <v>36</v>
       </c>
       <c r="I4" t="n">
         <v>0</v>
@@ -6889,10 +6889,10 @@
         <v>19</v>
       </c>
       <c r="D20" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E20" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F20" t="n">
         <v>0</v>
@@ -6901,7 +6901,7 @@
         <v>0</v>
       </c>
       <c r="H20" t="n">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="I20" t="n">
         <v>0</v>
@@ -6968,22 +6968,22 @@
         <v>2</v>
       </c>
       <c r="C21" t="n">
-        <v>9</v>
+        <v>16</v>
       </c>
       <c r="D21" t="n">
+        <v>11</v>
+      </c>
+      <c r="E21" t="n">
         <v>5</v>
       </c>
-      <c r="E21" t="n">
-        <v>4</v>
-      </c>
       <c r="F21" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G21" t="n">
         <v>0</v>
       </c>
       <c r="H21" t="n">
-        <v>20</v>
+        <v>35</v>
       </c>
       <c r="I21" t="n">
         <v>0</v>
@@ -7952,22 +7952,22 @@
         <v>0</v>
       </c>
       <c r="C33" t="n">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="D33" t="n">
         <v>0</v>
       </c>
       <c r="E33" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="F33" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G33" t="n">
         <v>0</v>
       </c>
       <c r="H33" t="n">
-        <v>18</v>
+        <v>30</v>
       </c>
       <c r="I33" t="n">
         <v>0</v>
@@ -8116,13 +8116,13 @@
         <v>0</v>
       </c>
       <c r="C35" t="n">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="D35" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E35" t="n">
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="F35" t="n">
         <v>0</v>
@@ -8131,7 +8131,7 @@
         <v>0</v>
       </c>
       <c r="H35" t="n">
-        <v>11</v>
+        <v>27</v>
       </c>
       <c r="I35" t="n">
         <v>0</v>
@@ -8772,22 +8772,22 @@
         <v>0</v>
       </c>
       <c r="C43" t="n">
-        <v>7</v>
+        <v>20</v>
       </c>
       <c r="D43" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E43" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="F43" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G43" t="n">
         <v>0</v>
       </c>
       <c r="H43" t="n">
-        <v>21</v>
+        <v>38</v>
       </c>
       <c r="I43" t="n">
         <v>0</v>
@@ -9343,25 +9343,25 @@
         </is>
       </c>
       <c r="B50" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C50" t="n">
-        <v>851</v>
+        <v>892</v>
       </c>
       <c r="D50" t="n">
-        <v>125</v>
+        <v>135</v>
       </c>
       <c r="E50" t="n">
-        <v>404</v>
+        <v>419</v>
       </c>
       <c r="F50" t="n">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="G50" t="n">
         <v>0</v>
       </c>
       <c r="H50" t="n">
-        <v>1466</v>
+        <v>1536</v>
       </c>
       <c r="I50" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Atualização automática LIRAa 2026-08-06 00:03 UTC
</commit_message>
<xml_diff>
--- a/data/LIRA_COMPLETO_latest.xlsx
+++ b/data/LIRA_COMPLETO_latest.xlsx
@@ -1774,10 +1774,10 @@
         <v>0</v>
       </c>
       <c r="C2" t="n">
-        <v>17</v>
+        <v>24</v>
       </c>
       <c r="D2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="E2" t="n">
         <v>3</v>
@@ -1789,7 +1789,7 @@
         <v>0</v>
       </c>
       <c r="H2" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="I2" t="n">
         <v>0</v>
@@ -2676,10 +2676,10 @@
         <v>6</v>
       </c>
       <c r="C13" t="n">
-        <v>174</v>
+        <v>181</v>
       </c>
       <c r="D13" t="n">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="E13" t="n">
         <v>33</v>
@@ -2691,7 +2691,7 @@
         <v>0</v>
       </c>
       <c r="H13" t="n">
-        <v>297</v>
+        <v>307</v>
       </c>
       <c r="I13" t="n">
         <v>0</v>
@@ -6394,10 +6394,10 @@
         <v>0</v>
       </c>
       <c r="C14" t="n">
-        <v>17</v>
+        <v>24</v>
       </c>
       <c r="D14" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="E14" t="n">
         <v>3</v>
@@ -6409,7 +6409,7 @@
         <v>0</v>
       </c>
       <c r="H14" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="I14" t="n">
         <v>0</v>
@@ -9346,10 +9346,10 @@
         <v>36</v>
       </c>
       <c r="C50" t="n">
-        <v>892</v>
+        <v>899</v>
       </c>
       <c r="D50" t="n">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="E50" t="n">
         <v>419</v>
@@ -9361,7 +9361,7 @@
         <v>0</v>
       </c>
       <c r="H50" t="n">
-        <v>1536</v>
+        <v>1546</v>
       </c>
       <c r="I50" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Atualização automática LIRAa 2026-08-06 11:16 UTC
</commit_message>
<xml_diff>
--- a/data/LIRA_COMPLETO_latest.xlsx
+++ b/data/LIRA_COMPLETO_latest.xlsx
@@ -808,10 +808,10 @@
         <v>0</v>
       </c>
       <c r="C5" t="n">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="D5" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E5" t="n">
         <v>5</v>
@@ -823,7 +823,7 @@
         <v>0</v>
       </c>
       <c r="H5" t="n">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="I5" t="n">
         <v>0</v>
@@ -1300,22 +1300,22 @@
         <v>0</v>
       </c>
       <c r="C11" t="n">
-        <v>18</v>
+        <v>34</v>
       </c>
       <c r="D11" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="E11" t="n">
+        <v>10</v>
+      </c>
+      <c r="F11" t="n">
         <v>5</v>
       </c>
-      <c r="F11" t="n">
-        <v>4</v>
-      </c>
       <c r="G11" t="n">
         <v>0</v>
       </c>
       <c r="H11" t="n">
-        <v>28</v>
+        <v>54</v>
       </c>
       <c r="I11" t="n">
         <v>0</v>
@@ -1546,22 +1546,22 @@
         <v>7</v>
       </c>
       <c r="C14" t="n">
-        <v>203</v>
+        <v>222</v>
       </c>
       <c r="D14" t="n">
-        <v>28</v>
+        <v>33</v>
       </c>
       <c r="E14" t="n">
-        <v>120</v>
+        <v>125</v>
       </c>
       <c r="F14" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="G14" t="n">
         <v>0</v>
       </c>
       <c r="H14" t="n">
-        <v>376</v>
+        <v>406</v>
       </c>
       <c r="I14" t="n">
         <v>0</v>
@@ -1856,13 +1856,13 @@
         <v>0</v>
       </c>
       <c r="C3" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="D3" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F3" t="n">
         <v>3</v>
@@ -1871,7 +1871,7 @@
         <v>0</v>
       </c>
       <c r="H3" t="n">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="I3" t="n">
         <v>0</v>
@@ -2184,13 +2184,13 @@
         <v>0</v>
       </c>
       <c r="C7" t="n">
-        <v>11</v>
+        <v>20</v>
       </c>
       <c r="D7" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="E7" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F7" t="n">
         <v>6</v>
@@ -2199,7 +2199,7 @@
         <v>0</v>
       </c>
       <c r="H7" t="n">
-        <v>23</v>
+        <v>39</v>
       </c>
       <c r="I7" t="n">
         <v>0</v>
@@ -2676,13 +2676,13 @@
         <v>6</v>
       </c>
       <c r="C13" t="n">
-        <v>181</v>
+        <v>192</v>
       </c>
       <c r="D13" t="n">
-        <v>70</v>
+        <v>77</v>
       </c>
       <c r="E13" t="n">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="F13" t="n">
         <v>23</v>
@@ -2691,7 +2691,7 @@
         <v>0</v>
       </c>
       <c r="H13" t="n">
-        <v>307</v>
+        <v>327</v>
       </c>
       <c r="I13" t="n">
         <v>0</v>
@@ -5656,10 +5656,10 @@
         <v>0</v>
       </c>
       <c r="C5" t="n">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="D5" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E5" t="n">
         <v>5</v>
@@ -5671,7 +5671,7 @@
         <v>0</v>
       </c>
       <c r="H5" t="n">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="I5" t="n">
         <v>0</v>
@@ -6148,22 +6148,22 @@
         <v>0</v>
       </c>
       <c r="C11" t="n">
-        <v>18</v>
+        <v>34</v>
       </c>
       <c r="D11" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="E11" t="n">
+        <v>10</v>
+      </c>
+      <c r="F11" t="n">
         <v>5</v>
       </c>
-      <c r="F11" t="n">
-        <v>4</v>
-      </c>
       <c r="G11" t="n">
         <v>0</v>
       </c>
       <c r="H11" t="n">
-        <v>28</v>
+        <v>54</v>
       </c>
       <c r="I11" t="n">
         <v>0</v>
@@ -6476,13 +6476,13 @@
         <v>0</v>
       </c>
       <c r="C15" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="D15" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E15" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F15" t="n">
         <v>3</v>
@@ -6491,7 +6491,7 @@
         <v>0</v>
       </c>
       <c r="H15" t="n">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="I15" t="n">
         <v>0</v>
@@ -6804,13 +6804,13 @@
         <v>0</v>
       </c>
       <c r="C19" t="n">
-        <v>11</v>
+        <v>20</v>
       </c>
       <c r="D19" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="E19" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F19" t="n">
         <v>6</v>
@@ -6819,7 +6819,7 @@
         <v>0</v>
       </c>
       <c r="H19" t="n">
-        <v>23</v>
+        <v>39</v>
       </c>
       <c r="I19" t="n">
         <v>0</v>
@@ -9346,22 +9346,22 @@
         <v>36</v>
       </c>
       <c r="C50" t="n">
-        <v>899</v>
+        <v>929</v>
       </c>
       <c r="D50" t="n">
-        <v>138</v>
+        <v>150</v>
       </c>
       <c r="E50" t="n">
-        <v>419</v>
+        <v>426</v>
       </c>
       <c r="F50" t="n">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="G50" t="n">
         <v>0</v>
       </c>
       <c r="H50" t="n">
-        <v>1546</v>
+        <v>1596</v>
       </c>
       <c r="I50" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Atualização automática LIRAa 2026-08-06 14:38 UTC
</commit_message>
<xml_diff>
--- a/data/LIRA_COMPLETO_latest.xlsx
+++ b/data/LIRA_COMPLETO_latest.xlsx
@@ -2013,29 +2013,29 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>AREA_1424</t>
+          <t>415 - CENTRO 1 - ESTRATO 2</t>
         </is>
       </c>
       <c r="B5" t="n">
         <v>0</v>
       </c>
       <c r="C5" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D5" t="n">
-        <v>0</v>
+        <v>23</v>
       </c>
       <c r="E5" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="F5" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="G5" t="n">
         <v>0</v>
       </c>
       <c r="H5" t="n">
-        <v>0</v>
+        <v>37</v>
       </c>
       <c r="I5" t="n">
         <v>0</v>
@@ -2600,7 +2600,7 @@
         <v>4</v>
       </c>
       <c r="E12" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F12" t="n">
         <v>0</v>
@@ -2609,7 +2609,7 @@
         <v>0</v>
       </c>
       <c r="H12" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="I12" t="n">
         <v>0</v>
@@ -2676,22 +2676,22 @@
         <v>6</v>
       </c>
       <c r="C13" t="n">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="D13" t="n">
-        <v>77</v>
+        <v>100</v>
       </c>
       <c r="E13" t="n">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="F13" t="n">
-        <v>23</v>
+        <v>30</v>
       </c>
       <c r="G13" t="n">
         <v>0</v>
       </c>
       <c r="H13" t="n">
-        <v>327</v>
+        <v>365</v>
       </c>
       <c r="I13" t="n">
         <v>0</v>
@@ -3256,7 +3256,7 @@
         <v>0</v>
       </c>
       <c r="K6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L6" t="n">
         <v>0</v>
@@ -3265,28 +3265,28 @@
         <v>0</v>
       </c>
       <c r="N6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O6" t="n">
         <v>0</v>
       </c>
       <c r="P6" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="Q6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R6" t="n">
         <v>0</v>
       </c>
       <c r="S6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T6" t="n">
         <v>0</v>
       </c>
       <c r="U6" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="V6" t="n">
         <v>0</v>
@@ -3994,7 +3994,7 @@
         <v>2</v>
       </c>
       <c r="K15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L15" t="n">
         <v>1</v>
@@ -4003,28 +4003,28 @@
         <v>0</v>
       </c>
       <c r="N15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O15" t="n">
         <v>0</v>
       </c>
       <c r="P15" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="Q15" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="R15" t="n">
         <v>0</v>
       </c>
       <c r="S15" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T15" t="n">
         <v>0</v>
       </c>
       <c r="U15" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="V15" t="n">
         <v>1</v>
@@ -4468,7 +4468,7 @@
         <v>0</v>
       </c>
       <c r="K5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L5" t="n">
         <v>0</v>
@@ -4483,10 +4483,10 @@
         <v>0</v>
       </c>
       <c r="P5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R5" t="n">
         <v>0</v>
@@ -4498,7 +4498,7 @@
         <v>0</v>
       </c>
       <c r="U5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V5" t="n">
         <v>0</v>
@@ -5206,7 +5206,7 @@
         <v>0</v>
       </c>
       <c r="K14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L14" t="n">
         <v>0</v>
@@ -5221,10 +5221,10 @@
         <v>0</v>
       </c>
       <c r="P14" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="Q14" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R14" t="n">
         <v>0</v>
@@ -5236,7 +5236,7 @@
         <v>0</v>
       </c>
       <c r="U14" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="V14" t="n">
         <v>0</v>
@@ -6633,29 +6633,29 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>AREA_1424</t>
+          <t>415 - CENTRO 1 - ESTRATO 2</t>
         </is>
       </c>
       <c r="B17" t="n">
         <v>0</v>
       </c>
       <c r="C17" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D17" t="n">
-        <v>0</v>
+        <v>23</v>
       </c>
       <c r="E17" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="F17" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="G17" t="n">
         <v>0</v>
       </c>
       <c r="H17" t="n">
-        <v>0</v>
+        <v>37</v>
       </c>
       <c r="I17" t="n">
         <v>0</v>
@@ -7220,7 +7220,7 @@
         <v>4</v>
       </c>
       <c r="E24" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F24" t="n">
         <v>0</v>
@@ -7229,7 +7229,7 @@
         <v>0</v>
       </c>
       <c r="H24" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="I24" t="n">
         <v>0</v>
@@ -7648,7 +7648,7 @@
         <v>0</v>
       </c>
       <c r="K29" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L29" t="n">
         <v>0</v>
@@ -7657,28 +7657,28 @@
         <v>0</v>
       </c>
       <c r="N29" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O29" t="n">
         <v>0</v>
       </c>
       <c r="P29" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="Q29" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R29" t="n">
         <v>0</v>
       </c>
       <c r="S29" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T29" t="n">
         <v>0</v>
       </c>
       <c r="U29" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="V29" t="n">
         <v>0</v>
@@ -8632,7 +8632,7 @@
         <v>0</v>
       </c>
       <c r="K41" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L41" t="n">
         <v>0</v>
@@ -8647,10 +8647,10 @@
         <v>0</v>
       </c>
       <c r="P41" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q41" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R41" t="n">
         <v>0</v>
@@ -8662,7 +8662,7 @@
         <v>0</v>
       </c>
       <c r="U41" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V41" t="n">
         <v>0</v>
@@ -9346,22 +9346,22 @@
         <v>36</v>
       </c>
       <c r="C50" t="n">
-        <v>929</v>
+        <v>931</v>
       </c>
       <c r="D50" t="n">
-        <v>150</v>
+        <v>173</v>
       </c>
       <c r="E50" t="n">
-        <v>426</v>
+        <v>432</v>
       </c>
       <c r="F50" t="n">
-        <v>91</v>
+        <v>98</v>
       </c>
       <c r="G50" t="n">
         <v>0</v>
       </c>
       <c r="H50" t="n">
-        <v>1596</v>
+        <v>1634</v>
       </c>
       <c r="I50" t="n">
         <v>0</v>
@@ -9370,7 +9370,7 @@
         <v>4</v>
       </c>
       <c r="K50" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="L50" t="n">
         <v>1</v>
@@ -9379,28 +9379,28 @@
         <v>0</v>
       </c>
       <c r="N50" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="O50" t="n">
         <v>0</v>
       </c>
       <c r="P50" t="n">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="Q50" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="R50" t="n">
         <v>0</v>
       </c>
       <c r="S50" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="T50" t="n">
         <v>0</v>
       </c>
       <c r="U50" t="n">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="V50" t="n">
         <v>1</v>

</xml_diff>

<commit_message>
Atualização automática LIRAa 2026-08-06 21:40 UTC
</commit_message>
<xml_diff>
--- a/data/LIRA_COMPLETO_latest.xlsx
+++ b/data/LIRA_COMPLETO_latest.xlsx
@@ -972,13 +972,13 @@
         <v>2</v>
       </c>
       <c r="C7" t="n">
-        <v>21</v>
+        <v>29</v>
       </c>
       <c r="D7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F7" t="n">
         <v>2</v>
@@ -987,7 +987,7 @@
         <v>0</v>
       </c>
       <c r="H7" t="n">
-        <v>25</v>
+        <v>35</v>
       </c>
       <c r="I7" t="n">
         <v>0</v>
@@ -1375,29 +1375,29 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>AREA_1419</t>
+          <t>410 - SALGADO FILHO - ESTRATO 1</t>
         </is>
       </c>
       <c r="B12" t="n">
         <v>0</v>
       </c>
       <c r="C12" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="D12" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E12" t="n">
         <v>0</v>
       </c>
       <c r="F12" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G12" t="n">
         <v>0</v>
       </c>
       <c r="H12" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="I12" t="n">
         <v>0</v>
@@ -1546,22 +1546,22 @@
         <v>7</v>
       </c>
       <c r="C14" t="n">
-        <v>222</v>
+        <v>237</v>
       </c>
       <c r="D14" t="n">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="E14" t="n">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="F14" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="G14" t="n">
         <v>0</v>
       </c>
       <c r="H14" t="n">
-        <v>406</v>
+        <v>425</v>
       </c>
       <c r="I14" t="n">
         <v>0</v>
@@ -2020,22 +2020,22 @@
         <v>0</v>
       </c>
       <c r="C5" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D5" t="n">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="E5" t="n">
         <v>5</v>
       </c>
       <c r="F5" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G5" t="n">
         <v>0</v>
       </c>
       <c r="H5" t="n">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="I5" t="n">
         <v>0</v>
@@ -2594,13 +2594,13 @@
         <v>0</v>
       </c>
       <c r="C12" t="n">
-        <v>21</v>
+        <v>34</v>
       </c>
       <c r="D12" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="E12" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="F12" t="n">
         <v>0</v>
@@ -2609,7 +2609,7 @@
         <v>0</v>
       </c>
       <c r="H12" t="n">
-        <v>29</v>
+        <v>49</v>
       </c>
       <c r="I12" t="n">
         <v>0</v>
@@ -2676,22 +2676,22 @@
         <v>6</v>
       </c>
       <c r="C13" t="n">
-        <v>194</v>
+        <v>208</v>
       </c>
       <c r="D13" t="n">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="E13" t="n">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="F13" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="G13" t="n">
         <v>0</v>
       </c>
       <c r="H13" t="n">
-        <v>365</v>
+        <v>389</v>
       </c>
       <c r="I13" t="n">
         <v>0</v>
@@ -3724,13 +3724,13 @@
         <v>0</v>
       </c>
       <c r="C12" t="n">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="D12" t="n">
         <v>2</v>
       </c>
       <c r="E12" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="F12" t="n">
         <v>0</v>
@@ -3739,7 +3739,7 @@
         <v>0</v>
       </c>
       <c r="H12" t="n">
-        <v>27</v>
+        <v>34</v>
       </c>
       <c r="I12" t="n">
         <v>0</v>
@@ -3970,13 +3970,13 @@
         <v>17</v>
       </c>
       <c r="C15" t="n">
-        <v>285</v>
+        <v>290</v>
       </c>
       <c r="D15" t="n">
         <v>18</v>
       </c>
       <c r="E15" t="n">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="F15" t="n">
         <v>19</v>
@@ -3985,7 +3985,7 @@
         <v>0</v>
       </c>
       <c r="H15" t="n">
-        <v>448</v>
+        <v>455</v>
       </c>
       <c r="I15" t="n">
         <v>0</v>
@@ -4936,13 +4936,13 @@
         <v>0</v>
       </c>
       <c r="C11" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="D11" t="n">
         <v>0</v>
       </c>
       <c r="E11" t="n">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="F11" t="n">
         <v>1</v>
@@ -4951,7 +4951,7 @@
         <v>0</v>
       </c>
       <c r="H11" t="n">
-        <v>16</v>
+        <v>25</v>
       </c>
       <c r="I11" t="n">
         <v>0</v>
@@ -5182,13 +5182,13 @@
         <v>6</v>
       </c>
       <c r="C14" t="n">
-        <v>230</v>
+        <v>233</v>
       </c>
       <c r="D14" t="n">
         <v>22</v>
       </c>
       <c r="E14" t="n">
-        <v>140</v>
+        <v>146</v>
       </c>
       <c r="F14" t="n">
         <v>23</v>
@@ -5197,7 +5197,7 @@
         <v>0</v>
       </c>
       <c r="H14" t="n">
-        <v>415</v>
+        <v>424</v>
       </c>
       <c r="I14" t="n">
         <v>0</v>
@@ -5820,13 +5820,13 @@
         <v>2</v>
       </c>
       <c r="C7" t="n">
-        <v>21</v>
+        <v>29</v>
       </c>
       <c r="D7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F7" t="n">
         <v>2</v>
@@ -5835,7 +5835,7 @@
         <v>0</v>
       </c>
       <c r="H7" t="n">
-        <v>25</v>
+        <v>35</v>
       </c>
       <c r="I7" t="n">
         <v>0</v>
@@ -6223,29 +6223,29 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>AREA_1419</t>
+          <t>410 - SALGADO FILHO - ESTRATO 1</t>
         </is>
       </c>
       <c r="B12" t="n">
         <v>0</v>
       </c>
       <c r="C12" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="D12" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E12" t="n">
         <v>0</v>
       </c>
       <c r="F12" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G12" t="n">
         <v>0</v>
       </c>
       <c r="H12" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="I12" t="n">
         <v>0</v>
@@ -6640,22 +6640,22 @@
         <v>0</v>
       </c>
       <c r="C17" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D17" t="n">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="E17" t="n">
         <v>5</v>
       </c>
       <c r="F17" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G17" t="n">
         <v>0</v>
       </c>
       <c r="H17" t="n">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="I17" t="n">
         <v>0</v>
@@ -7214,13 +7214,13 @@
         <v>0</v>
       </c>
       <c r="C24" t="n">
-        <v>21</v>
+        <v>34</v>
       </c>
       <c r="D24" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="E24" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="F24" t="n">
         <v>0</v>
@@ -7229,7 +7229,7 @@
         <v>0</v>
       </c>
       <c r="H24" t="n">
-        <v>29</v>
+        <v>49</v>
       </c>
       <c r="I24" t="n">
         <v>0</v>
@@ -8116,13 +8116,13 @@
         <v>0</v>
       </c>
       <c r="C35" t="n">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="D35" t="n">
         <v>2</v>
       </c>
       <c r="E35" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="F35" t="n">
         <v>0</v>
@@ -8131,7 +8131,7 @@
         <v>0</v>
       </c>
       <c r="H35" t="n">
-        <v>27</v>
+        <v>34</v>
       </c>
       <c r="I35" t="n">
         <v>0</v>
@@ -9100,13 +9100,13 @@
         <v>0</v>
       </c>
       <c r="C47" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="D47" t="n">
         <v>0</v>
       </c>
       <c r="E47" t="n">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="F47" t="n">
         <v>1</v>
@@ -9115,7 +9115,7 @@
         <v>0</v>
       </c>
       <c r="H47" t="n">
-        <v>16</v>
+        <v>25</v>
       </c>
       <c r="I47" t="n">
         <v>0</v>
@@ -9346,22 +9346,22 @@
         <v>36</v>
       </c>
       <c r="C50" t="n">
-        <v>931</v>
+        <v>968</v>
       </c>
       <c r="D50" t="n">
-        <v>173</v>
+        <v>181</v>
       </c>
       <c r="E50" t="n">
-        <v>432</v>
+        <v>444</v>
       </c>
       <c r="F50" t="n">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="G50" t="n">
         <v>0</v>
       </c>
       <c r="H50" t="n">
-        <v>1634</v>
+        <v>1693</v>
       </c>
       <c r="I50" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Atualização automática LIRAa 2026-08-07 01:45 UTC
</commit_message>
<xml_diff>
--- a/data/LIRA_COMPLETO_latest.xlsx
+++ b/data/LIRA_COMPLETO_latest.xlsx
@@ -972,7 +972,7 @@
         <v>2</v>
       </c>
       <c r="C7" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D7" t="n">
         <v>2</v>
@@ -987,7 +987,7 @@
         <v>0</v>
       </c>
       <c r="H7" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="I7" t="n">
         <v>0</v>
@@ -1546,7 +1546,7 @@
         <v>7</v>
       </c>
       <c r="C14" t="n">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="D14" t="n">
         <v>35</v>
@@ -1561,7 +1561,7 @@
         <v>0</v>
       </c>
       <c r="H14" t="n">
-        <v>425</v>
+        <v>426</v>
       </c>
       <c r="I14" t="n">
         <v>0</v>
@@ -5820,7 +5820,7 @@
         <v>2</v>
       </c>
       <c r="C7" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D7" t="n">
         <v>2</v>
@@ -5835,7 +5835,7 @@
         <v>0</v>
       </c>
       <c r="H7" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="I7" t="n">
         <v>0</v>
@@ -9346,7 +9346,7 @@
         <v>36</v>
       </c>
       <c r="C50" t="n">
-        <v>968</v>
+        <v>969</v>
       </c>
       <c r="D50" t="n">
         <v>181</v>
@@ -9361,7 +9361,7 @@
         <v>0</v>
       </c>
       <c r="H50" t="n">
-        <v>1693</v>
+        <v>1694</v>
       </c>
       <c r="I50" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Atualização automática LIRAa 2026-08-07 09:55 UTC
</commit_message>
<xml_diff>
--- a/data/LIRA_COMPLETO_latest.xlsx
+++ b/data/LIRA_COMPLETO_latest.xlsx
@@ -1382,22 +1382,22 @@
         <v>0</v>
       </c>
       <c r="C12" t="n">
-        <v>7</v>
+        <v>15</v>
       </c>
       <c r="D12" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E12" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="F12" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="G12" t="n">
         <v>0</v>
       </c>
       <c r="H12" t="n">
-        <v>9</v>
+        <v>27</v>
       </c>
       <c r="I12" t="n">
         <v>0</v>
@@ -1546,22 +1546,22 @@
         <v>7</v>
       </c>
       <c r="C14" t="n">
-        <v>238</v>
+        <v>246</v>
       </c>
       <c r="D14" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="E14" t="n">
-        <v>126</v>
+        <v>131</v>
       </c>
       <c r="F14" t="n">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="G14" t="n">
         <v>0</v>
       </c>
       <c r="H14" t="n">
-        <v>426</v>
+        <v>444</v>
       </c>
       <c r="I14" t="n">
         <v>0</v>
@@ -6230,22 +6230,22 @@
         <v>0</v>
       </c>
       <c r="C12" t="n">
-        <v>7</v>
+        <v>15</v>
       </c>
       <c r="D12" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E12" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="F12" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="G12" t="n">
         <v>0</v>
       </c>
       <c r="H12" t="n">
-        <v>9</v>
+        <v>27</v>
       </c>
       <c r="I12" t="n">
         <v>0</v>
@@ -9346,22 +9346,22 @@
         <v>36</v>
       </c>
       <c r="C50" t="n">
-        <v>969</v>
+        <v>977</v>
       </c>
       <c r="D50" t="n">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="E50" t="n">
-        <v>444</v>
+        <v>449</v>
       </c>
       <c r="F50" t="n">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="G50" t="n">
         <v>0</v>
       </c>
       <c r="H50" t="n">
-        <v>1694</v>
+        <v>1712</v>
       </c>
       <c r="I50" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Atualização automática LIRAa 2026-08-07 16:56 UTC
</commit_message>
<xml_diff>
--- a/data/LIRA_COMPLETO_latest.xlsx
+++ b/data/LIRA_COMPLETO_latest.xlsx
@@ -1382,22 +1382,22 @@
         <v>0</v>
       </c>
       <c r="C12" t="n">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="D12" t="n">
         <v>2</v>
       </c>
       <c r="E12" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F12" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G12" t="n">
         <v>0</v>
       </c>
       <c r="H12" t="n">
-        <v>27</v>
+        <v>35</v>
       </c>
       <c r="I12" t="n">
         <v>0</v>
@@ -1546,22 +1546,22 @@
         <v>7</v>
       </c>
       <c r="C14" t="n">
-        <v>246</v>
+        <v>252</v>
       </c>
       <c r="D14" t="n">
         <v>36</v>
       </c>
       <c r="E14" t="n">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="F14" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="G14" t="n">
         <v>0</v>
       </c>
       <c r="H14" t="n">
-        <v>444</v>
+        <v>452</v>
       </c>
       <c r="I14" t="n">
         <v>0</v>
@@ -4936,13 +4936,13 @@
         <v>0</v>
       </c>
       <c r="C11" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="D11" t="n">
         <v>0</v>
       </c>
       <c r="E11" t="n">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="F11" t="n">
         <v>1</v>
@@ -4951,7 +4951,7 @@
         <v>0</v>
       </c>
       <c r="H11" t="n">
-        <v>25</v>
+        <v>31</v>
       </c>
       <c r="I11" t="n">
         <v>0</v>
@@ -5182,13 +5182,13 @@
         <v>6</v>
       </c>
       <c r="C14" t="n">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="D14" t="n">
         <v>22</v>
       </c>
       <c r="E14" t="n">
-        <v>146</v>
+        <v>150</v>
       </c>
       <c r="F14" t="n">
         <v>23</v>
@@ -5197,7 +5197,7 @@
         <v>0</v>
       </c>
       <c r="H14" t="n">
-        <v>424</v>
+        <v>430</v>
       </c>
       <c r="I14" t="n">
         <v>0</v>
@@ -6230,22 +6230,22 @@
         <v>0</v>
       </c>
       <c r="C12" t="n">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="D12" t="n">
         <v>2</v>
       </c>
       <c r="E12" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F12" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G12" t="n">
         <v>0</v>
       </c>
       <c r="H12" t="n">
-        <v>27</v>
+        <v>35</v>
       </c>
       <c r="I12" t="n">
         <v>0</v>
@@ -9100,13 +9100,13 @@
         <v>0</v>
       </c>
       <c r="C47" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="D47" t="n">
         <v>0</v>
       </c>
       <c r="E47" t="n">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="F47" t="n">
         <v>1</v>
@@ -9115,7 +9115,7 @@
         <v>0</v>
       </c>
       <c r="H47" t="n">
-        <v>25</v>
+        <v>31</v>
       </c>
       <c r="I47" t="n">
         <v>0</v>
@@ -9346,22 +9346,22 @@
         <v>36</v>
       </c>
       <c r="C50" t="n">
-        <v>977</v>
+        <v>985</v>
       </c>
       <c r="D50" t="n">
         <v>182</v>
       </c>
       <c r="E50" t="n">
-        <v>449</v>
+        <v>454</v>
       </c>
       <c r="F50" t="n">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="G50" t="n">
         <v>0</v>
       </c>
       <c r="H50" t="n">
-        <v>1712</v>
+        <v>1726</v>
       </c>
       <c r="I50" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Atualização automática LIRAa 2026-08-10 16:43 UTC
</commit_message>
<xml_diff>
--- a/data/LIRA_COMPLETO_latest.xlsx
+++ b/data/LIRA_COMPLETO_latest.xlsx
@@ -756,7 +756,7 @@
         <v>0</v>
       </c>
       <c r="M4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N4" t="n">
         <v>0</v>
@@ -765,10 +765,10 @@
         <v>0</v>
       </c>
       <c r="P4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R4" t="n">
         <v>0</v>
@@ -780,7 +780,7 @@
         <v>0</v>
       </c>
       <c r="U4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V4" t="n">
         <v>0</v>
@@ -1576,7 +1576,7 @@
         <v>0</v>
       </c>
       <c r="M14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N14" t="n">
         <v>0</v>
@@ -1585,10 +1585,10 @@
         <v>0</v>
       </c>
       <c r="P14" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="Q14" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R14" t="n">
         <v>0</v>
@@ -1600,7 +1600,7 @@
         <v>0</v>
       </c>
       <c r="U14" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="V14" t="n">
         <v>0</v>
@@ -2372,7 +2372,7 @@
         <v>0</v>
       </c>
       <c r="K9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L9" t="n">
         <v>0</v>
@@ -2387,10 +2387,10 @@
         <v>0</v>
       </c>
       <c r="P9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R9" t="n">
         <v>0</v>
@@ -2402,7 +2402,7 @@
         <v>0</v>
       </c>
       <c r="U9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V9" t="n">
         <v>0</v>
@@ -2700,7 +2700,7 @@
         <v>1</v>
       </c>
       <c r="K13" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L13" t="n">
         <v>0</v>
@@ -2715,10 +2715,10 @@
         <v>0</v>
       </c>
       <c r="P13" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="Q13" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="R13" t="n">
         <v>0</v>
@@ -2730,7 +2730,7 @@
         <v>0</v>
       </c>
       <c r="U13" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="V13" t="n">
         <v>0</v>
@@ -3010,7 +3010,7 @@
         <v>0</v>
       </c>
       <c r="K3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L3" t="n">
         <v>0</v>
@@ -3025,10 +3025,10 @@
         <v>0</v>
       </c>
       <c r="P3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R3" t="n">
         <v>0</v>
@@ -3040,7 +3040,7 @@
         <v>0</v>
       </c>
       <c r="U3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V3" t="n">
         <v>0</v>
@@ -3511,13 +3511,13 @@
         <v>0</v>
       </c>
       <c r="N9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O9" t="n">
         <v>0</v>
       </c>
       <c r="P9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q9" t="n">
         <v>0</v>
@@ -3526,13 +3526,13 @@
         <v>0</v>
       </c>
       <c r="S9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T9" t="n">
         <v>0</v>
       </c>
       <c r="U9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V9" t="n">
         <v>0</v>
@@ -3541,13 +3541,13 @@
         <v>0</v>
       </c>
       <c r="X9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Y9" t="n">
         <v>0</v>
       </c>
       <c r="Z9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="10">
@@ -3724,13 +3724,13 @@
         <v>0</v>
       </c>
       <c r="C12" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D12" t="n">
         <v>2</v>
       </c>
       <c r="E12" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="F12" t="n">
         <v>0</v>
@@ -3839,13 +3839,13 @@
         <v>0</v>
       </c>
       <c r="N13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O13" t="n">
         <v>0</v>
       </c>
       <c r="P13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q13" t="n">
         <v>0</v>
@@ -3854,13 +3854,13 @@
         <v>0</v>
       </c>
       <c r="S13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T13" t="n">
         <v>0</v>
       </c>
       <c r="U13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V13" t="n">
         <v>0</v>
@@ -3970,13 +3970,13 @@
         <v>17</v>
       </c>
       <c r="C15" t="n">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="D15" t="n">
         <v>18</v>
       </c>
       <c r="E15" t="n">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="F15" t="n">
         <v>19</v>
@@ -3994,7 +3994,7 @@
         <v>2</v>
       </c>
       <c r="K15" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L15" t="n">
         <v>1</v>
@@ -4003,28 +4003,28 @@
         <v>0</v>
       </c>
       <c r="N15" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="O15" t="n">
         <v>0</v>
       </c>
       <c r="P15" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q15" t="n">
         <v>7</v>
       </c>
-      <c r="Q15" t="n">
-        <v>6</v>
-      </c>
       <c r="R15" t="n">
         <v>0</v>
       </c>
       <c r="S15" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="T15" t="n">
         <v>0</v>
       </c>
       <c r="U15" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="V15" t="n">
         <v>1</v>
@@ -4033,13 +4033,13 @@
         <v>0</v>
       </c>
       <c r="X15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Y15" t="n">
         <v>0</v>
       </c>
       <c r="Z15" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
   </sheetData>
@@ -5604,7 +5604,7 @@
         <v>0</v>
       </c>
       <c r="M4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N4" t="n">
         <v>0</v>
@@ -5613,10 +5613,10 @@
         <v>0</v>
       </c>
       <c r="P4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R4" t="n">
         <v>0</v>
@@ -5628,7 +5628,7 @@
         <v>0</v>
       </c>
       <c r="U4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V4" t="n">
         <v>0</v>
@@ -6992,7 +6992,7 @@
         <v>0</v>
       </c>
       <c r="K21" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L21" t="n">
         <v>0</v>
@@ -7007,10 +7007,10 @@
         <v>0</v>
       </c>
       <c r="P21" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q21" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R21" t="n">
         <v>0</v>
@@ -7022,7 +7022,7 @@
         <v>0</v>
       </c>
       <c r="U21" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V21" t="n">
         <v>0</v>
@@ -7402,7 +7402,7 @@
         <v>0</v>
       </c>
       <c r="K26" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L26" t="n">
         <v>0</v>
@@ -7417,10 +7417,10 @@
         <v>0</v>
       </c>
       <c r="P26" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q26" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R26" t="n">
         <v>0</v>
@@ -7432,7 +7432,7 @@
         <v>0</v>
       </c>
       <c r="U26" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V26" t="n">
         <v>0</v>
@@ -7903,13 +7903,13 @@
         <v>0</v>
       </c>
       <c r="N32" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O32" t="n">
         <v>0</v>
       </c>
       <c r="P32" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q32" t="n">
         <v>0</v>
@@ -7918,13 +7918,13 @@
         <v>0</v>
       </c>
       <c r="S32" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T32" t="n">
         <v>0</v>
       </c>
       <c r="U32" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V32" t="n">
         <v>0</v>
@@ -7933,13 +7933,13 @@
         <v>0</v>
       </c>
       <c r="X32" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Y32" t="n">
         <v>0</v>
       </c>
       <c r="Z32" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="33">
@@ -8116,13 +8116,13 @@
         <v>0</v>
       </c>
       <c r="C35" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D35" t="n">
         <v>2</v>
       </c>
       <c r="E35" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="F35" t="n">
         <v>0</v>
@@ -8231,13 +8231,13 @@
         <v>0</v>
       </c>
       <c r="N36" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O36" t="n">
         <v>0</v>
       </c>
       <c r="P36" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q36" t="n">
         <v>0</v>
@@ -8246,13 +8246,13 @@
         <v>0</v>
       </c>
       <c r="S36" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T36" t="n">
         <v>0</v>
       </c>
       <c r="U36" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V36" t="n">
         <v>0</v>
@@ -9346,13 +9346,13 @@
         <v>36</v>
       </c>
       <c r="C50" t="n">
-        <v>985</v>
+        <v>984</v>
       </c>
       <c r="D50" t="n">
         <v>182</v>
       </c>
       <c r="E50" t="n">
-        <v>454</v>
+        <v>455</v>
       </c>
       <c r="F50" t="n">
         <v>105</v>
@@ -9370,37 +9370,37 @@
         <v>4</v>
       </c>
       <c r="K50" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="L50" t="n">
         <v>1</v>
       </c>
       <c r="M50" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N50" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="O50" t="n">
         <v>0</v>
       </c>
       <c r="P50" t="n">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="Q50" t="n">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="R50" t="n">
         <v>0</v>
       </c>
       <c r="S50" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="T50" t="n">
         <v>0</v>
       </c>
       <c r="U50" t="n">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="V50" t="n">
         <v>1</v>
@@ -9409,13 +9409,13 @@
         <v>0</v>
       </c>
       <c r="X50" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Y50" t="n">
         <v>0</v>
       </c>
       <c r="Z50" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualização automática LIRAa 2026-08-10 17:53 UTC
</commit_message>
<xml_diff>
--- a/data/LIRA_COMPLETO_latest.xlsx
+++ b/data/LIRA_COMPLETO_latest.xlsx
@@ -3347,13 +3347,13 @@
         <v>0</v>
       </c>
       <c r="N7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O7" t="n">
         <v>0</v>
       </c>
       <c r="P7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q7" t="n">
         <v>0</v>
@@ -3362,13 +3362,13 @@
         <v>0</v>
       </c>
       <c r="S7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T7" t="n">
         <v>0</v>
       </c>
       <c r="U7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V7" t="n">
         <v>0</v>
@@ -4003,13 +4003,13 @@
         <v>0</v>
       </c>
       <c r="N15" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="O15" t="n">
         <v>0</v>
       </c>
       <c r="P15" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="Q15" t="n">
         <v>7</v>
@@ -4018,13 +4018,13 @@
         <v>0</v>
       </c>
       <c r="S15" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T15" t="n">
         <v>0</v>
       </c>
       <c r="U15" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="V15" t="n">
         <v>1</v>
@@ -7739,13 +7739,13 @@
         <v>0</v>
       </c>
       <c r="N30" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O30" t="n">
         <v>0</v>
       </c>
       <c r="P30" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q30" t="n">
         <v>0</v>
@@ -7754,13 +7754,13 @@
         <v>0</v>
       </c>
       <c r="S30" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T30" t="n">
         <v>0</v>
       </c>
       <c r="U30" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V30" t="n">
         <v>0</v>
@@ -9379,13 +9379,13 @@
         <v>1</v>
       </c>
       <c r="N50" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="O50" t="n">
         <v>0</v>
       </c>
       <c r="P50" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="Q50" t="n">
         <v>16</v>
@@ -9394,13 +9394,13 @@
         <v>0</v>
       </c>
       <c r="S50" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="T50" t="n">
         <v>0</v>
       </c>
       <c r="U50" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="V50" t="n">
         <v>1</v>

</xml_diff>